<commit_message>
revised: Buffett Analysis Excel Template
</commit_message>
<xml_diff>
--- a/investment_analysis_framework_prompt/Buffett_Analysis_Template.xlsx
+++ b/investment_analysis_framework_prompt/Buffett_Analysis_Template.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="610" uniqueCount="417">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="632" uniqueCount="432">
   <si>
     <t xml:space="preserve">═══════════════════════════════════════════════════════════</t>
   </si>
@@ -940,6 +940,51 @@
   </si>
   <si>
     <t xml:space="preserve">Analyst Consensus %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">STEP 3B: BUFFETT-PURE REVERSE DCF — Implied Owner Earnings (OEPS) CAGR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Note: EPS can be flattered by under-investment or leverage. Owner Earnings strips this out. If OEPS-implied growth &gt;&gt; EPS-implied growth, the business is capital-hungry and EPS understates the true hurdle.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current OEPS (₹)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Current P/OE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TERMINAL P/OE SCENARIOS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mature (13x)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Market (17x)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compounder (22x)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Terminal P/OE Value</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implied OEPS CAGR — at Market P/OE (17x)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THE DIVERGENCE TEST — EPS vs OEPS (10Y, 10% return, same 20x terminal multiple)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implied EPS CAGR (from EPS block above)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Implied OEPS CAGR (same 20x)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Gap (OEPS − EPS), percentage points</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reading: Gap ≈ 0 → EPS reliable (asset-light). Gap large &amp; positive (OEPS hurdle higher) → capital-hungry, EPS flatters; trust OEPS. Sign depends on Maintenance CapEx % in Sheet 16 — set it ≥100% of D&amp;A for capital-heavy firms to make this test meaningful.</t>
   </si>
   <si>
     <t xml:space="preserve">SECTION 14B: P/B SCENARIO RETURN ANALYSIS</t>
@@ -1305,10 +1350,10 @@
     <numFmt numFmtId="171" formatCode="0.00%"/>
     <numFmt numFmtId="172" formatCode="0.0000"/>
     <numFmt numFmtId="173" formatCode="\₹#,##0.00"/>
-    <numFmt numFmtId="174" formatCode="\₹#,##0"/>
-    <numFmt numFmtId="175" formatCode="0.0\:1"/>
-    <numFmt numFmtId="176" formatCode="0"/>
-    <numFmt numFmtId="177" formatCode="0.0"/>
+    <numFmt numFmtId="174" formatCode="0.0"/>
+    <numFmt numFmtId="175" formatCode="\₹#,##0"/>
+    <numFmt numFmtId="176" formatCode="0.0\:1"/>
+    <numFmt numFmtId="177" formatCode="0"/>
   </numFmts>
   <fonts count="18">
     <font>
@@ -1520,7 +1565,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="52">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1645,6 +1690,30 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="174" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="173" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1657,15 +1726,15 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="175" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="175" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="174" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="175" fontId="5" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1677,7 +1746,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="175" fontId="16" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="176" fontId="16" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1693,15 +1762,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="176" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="177" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="177" fontId="16" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="174" fontId="16" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="17" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="17" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2603,9 +2672,9 @@
       <c r="A26" s="17" t="s">
         <v>273</v>
       </c>
-      <c r="B26" s="12" t="e">
-        <f aca="false">IF(B25=0,"-",(B25-$B$11)/B25)</f>
-        <v>#VALUE!</v>
+      <c r="B26" s="12" t="str">
+        <f aca="false">IFERROR((B25-$B$11)/B25,"-")</f>
+        <v>-</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2887,9 +2956,9 @@
       <c r="A44" s="17" t="s">
         <v>273</v>
       </c>
-      <c r="B44" s="12" t="e">
-        <f aca="false">IF(B43=0,"-",(B43-$C$11)/B43)</f>
-        <v>#VALUE!</v>
+      <c r="B44" s="12" t="str">
+        <f aca="false">IFERROR((B43-$C$11)/B43,"-")</f>
+        <v>-</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3171,9 +3240,9 @@
       <c r="A62" s="17" t="s">
         <v>273</v>
       </c>
-      <c r="B62" s="12" t="e">
-        <f aca="false">IF(B61=0,"-",(B61-$D$11)/B61)</f>
-        <v>#VALUE!</v>
+      <c r="B62" s="12" t="str">
+        <f aca="false">IFERROR((B61-$D$11)/B61,"-")</f>
+        <v>-</v>
       </c>
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3205,7 +3274,7 @@
     <tabColor rgb="FFFF0000"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="35"/>
@@ -3283,7 +3352,10 @@
       <c r="D9" s="29" t="n">
         <v>28</v>
       </c>
-      <c r="E9" s="29"/>
+      <c r="E9" s="29" t="n">
+        <f aca="false">'1. Inputs'!B63</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
@@ -3556,8 +3628,8 @@
         <v>298</v>
       </c>
       <c r="B42" s="30" t="n">
-        <f aca="false">'1. Inputs'!B62</f>
-        <v>0</v>
+        <f aca="false">'1. Inputs'!B72</f>
+        <v>11</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3594,6 +3666,169 @@
       <c r="B46" s="30" t="n">
         <f aca="false">'1. Inputs'!B76</f>
         <v>0</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="31" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="2" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="31" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="B52" s="1" t="str">
+        <f aca="false">'16. Owner Earnings'!L11</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A53" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="B53" s="32" t="str">
+        <f aca="false">IF(OR(B52="-",B52=0),"-",$B$4/B52)</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A55" s="31" t="s">
+        <v>305</v>
+      </c>
+      <c r="B55" s="33" t="s">
+        <v>306</v>
+      </c>
+      <c r="C55" s="33" t="s">
+        <v>307</v>
+      </c>
+      <c r="D55" s="33" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A56" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="B56" s="34" t="n">
+        <v>13</v>
+      </c>
+      <c r="C56" s="34" t="n">
+        <v>17</v>
+      </c>
+      <c r="D56" s="34" t="n">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A58" s="31" t="s">
+        <v>310</v>
+      </c>
+      <c r="B58" s="33" t="s">
+        <v>288</v>
+      </c>
+      <c r="C58" s="33" t="s">
+        <v>289</v>
+      </c>
+      <c r="D58" s="33" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A59" s="2" t="s">
+        <v>291</v>
+      </c>
+      <c r="B59" s="35" t="str">
+        <f aca="false">IFERROR((($B$4*(1+10/100)^5/$C$56)/$B$52)^(1/5)-1,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="C59" s="35" t="str">
+        <f aca="false">IFERROR((($B$4*(1+15/100)^5/$C$56)/$B$52)^(1/5)-1,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="D59" s="35" t="str">
+        <f aca="false">IFERROR((($B$4*(1+20/100)^5/$C$56)/$B$52)^(1/5)-1,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="2" t="s">
+        <v>292</v>
+      </c>
+      <c r="B60" s="35" t="str">
+        <f aca="false">IFERROR((($B$4*(1+10/100)^10/$C$56)/$B$52)^(1/10)-1,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="C60" s="35" t="str">
+        <f aca="false">IFERROR((($B$4*(1+15/100)^10/$C$56)/$B$52)^(1/10)-1,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="D60" s="35" t="str">
+        <f aca="false">IFERROR((($B$4*(1+20/100)^10/$C$56)/$B$52)^(1/10)-1,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A61" s="2" t="s">
+        <v>293</v>
+      </c>
+      <c r="B61" s="35" t="str">
+        <f aca="false">IFERROR((($B$4*(1+10/100)^15/$C$56)/$B$52)^(1/15)-1,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="C61" s="35" t="str">
+        <f aca="false">IFERROR((($B$4*(1+15/100)^15/$C$56)/$B$52)^(1/15)-1,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="D61" s="35" t="str">
+        <f aca="false">IFERROR((($B$4*(1+20/100)^15/$C$56)/$B$52)^(1/15)-1,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A63" s="31" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A64" s="1" t="s">
+        <v>312</v>
+      </c>
+      <c r="B64" s="35" t="str">
+        <f aca="false">B20</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A65" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="B65" s="35" t="str">
+        <f aca="false">IFERROR((($B$4*(1+10/100)^10/$C$9)/$B$52)^(1/10)-1,"-")</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A66" s="1" t="s">
+        <v>314</v>
+      </c>
+      <c r="B66" s="36" t="str">
+        <f aca="false">IF(OR(B64="-",B65="-"),"-",(B65-B64)*100)</f>
+        <v>-</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A67" s="2" t="s">
+        <v>315</v>
       </c>
     </row>
   </sheetData>
@@ -3625,7 +3860,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>301</v>
+        <v>316</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -3639,10 +3874,10 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>302</v>
+        <v>317</v>
       </c>
       <c r="B4" s="11" t="n">
-        <f aca="false">'1. Inputs'!L38</f>
+        <f aca="false">'1. Inputs'!L39</f>
         <v>0</v>
       </c>
     </row>
@@ -3657,7 +3892,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>303</v>
+        <v>318</v>
       </c>
       <c r="B6" s="14" t="str">
         <f aca="false">IF(B4=0,"-",B5/B4)</f>
@@ -3678,7 +3913,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>304</v>
+        <v>319</v>
       </c>
       <c r="B9" s="12" t="n">
         <f aca="false">B7/100*B8/100</f>
@@ -3687,52 +3922,52 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>305</v>
+        <v>320</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>306</v>
+        <v>321</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>307</v>
+        <v>322</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>308</v>
+        <v>323</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>309</v>
-      </c>
-      <c r="B12" s="31" t="n">
+        <v>324</v>
+      </c>
+      <c r="B12" s="37" t="n">
         <f aca="false">B4*(1+B9)^5</f>
         <v>0</v>
       </c>
-      <c r="C12" s="31" t="n">
+      <c r="C12" s="37" t="n">
         <f aca="false">B4*(1+B9)^7</f>
         <v>0</v>
       </c>
-      <c r="D12" s="31" t="n">
+      <c r="D12" s="37" t="n">
         <f aca="false">B4*(1+B9)^10</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>310</v>
+        <v>325</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>311</v>
+        <v>326</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="D14" s="6" t="s">
-        <v>313</v>
+        <v>328</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
-        <v>314</v>
+        <v>329</v>
       </c>
       <c r="B15" s="12" t="str">
         <f aca="false">IFERROR((B12*B6/B5)^(1/5)-1,"-")</f>
@@ -3749,7 +3984,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="17" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
       <c r="B16" s="12" t="str">
         <f aca="false">IFERROR((B12*0.75*B6/B5)^(1/5)-1,"-")</f>
@@ -3766,7 +4001,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>316</v>
+        <v>331</v>
       </c>
       <c r="B17" s="12" t="str">
         <f aca="false">IFERROR((B12*0.5*B6/B5)^(1/5)-1,"-")</f>
@@ -3783,7 +4018,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="17" t="s">
-        <v>317</v>
+        <v>332</v>
       </c>
       <c r="B18" s="12" t="str">
         <f aca="false">IFERROR((B12*B22/B5)^(1/5)-1,"-")</f>
@@ -3800,7 +4035,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
-        <v>318</v>
+        <v>333</v>
       </c>
       <c r="B19" s="12" t="str">
         <f aca="false">IFERROR((B12*B23/B5)^(1/5)-1,"-")</f>
@@ -3817,7 +4052,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>319</v>
+        <v>334</v>
       </c>
       <c r="B20" s="12" t="str">
         <f aca="false">IFERROR((B12*1/B5)^(1/5)-1,"-")</f>
@@ -3833,16 +4068,16 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="32" t="s">
-        <v>320</v>
-      </c>
-      <c r="B22" s="33"/>
+      <c r="A22" s="38" t="s">
+        <v>335</v>
+      </c>
+      <c r="B22" s="39"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="32" t="s">
-        <v>321</v>
-      </c>
-      <c r="B23" s="33"/>
+      <c r="A23" s="38" t="s">
+        <v>336</v>
+      </c>
+      <c r="B23" s="39"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -3873,7 +4108,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>322</v>
+        <v>337</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -3882,138 +4117,138 @@
     </row>
     <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>323</v>
+        <v>338</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>324</v>
+        <v>339</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>325</v>
+        <v>340</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>326</v>
+        <v>341</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>327</v>
+        <v>342</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="32" t="s">
-        <v>328</v>
-      </c>
-      <c r="B4" s="34"/>
+      <c r="A4" s="38" t="s">
+        <v>343</v>
+      </c>
+      <c r="B4" s="40"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
         <v>201</v>
       </c>
-      <c r="B5" s="35" t="n">
+      <c r="B5" s="41" t="n">
         <f aca="false">'1. Inputs'!B4</f>
         <v>0</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>329</v>
-      </c>
-      <c r="B7" s="36" t="n">
+        <v>344</v>
+      </c>
+      <c r="B7" s="42" t="n">
         <f aca="false">B4*0.5</f>
         <v>0</v>
       </c>
-      <c r="C7" s="36" t="n">
+      <c r="C7" s="42" t="n">
         <f aca="false">B4*0.7</f>
         <v>0</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>330</v>
-      </c>
-      <c r="E7" s="37" t="str">
+        <v>345</v>
+      </c>
+      <c r="E7" s="43" t="str">
         <f aca="false">IF(AND(B5&gt;=B7,B5&lt;C7),"◄ CURRENT","")</f>
         <v/>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>331</v>
-      </c>
-      <c r="B8" s="36" t="n">
+        <v>346</v>
+      </c>
+      <c r="B8" s="42" t="n">
         <f aca="false">B4*0.7</f>
         <v>0</v>
       </c>
-      <c r="C8" s="36" t="n">
+      <c r="C8" s="42" t="n">
         <f aca="false">B4*0.9</f>
         <v>0</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>332</v>
-      </c>
-      <c r="E8" s="37" t="str">
+        <v>347</v>
+      </c>
+      <c r="E8" s="43" t="str">
         <f aca="false">IF(AND(B5&gt;=B8,B5&lt;C8),"◄ CURRENT","")</f>
         <v/>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>333</v>
-      </c>
-      <c r="B9" s="36" t="n">
+        <v>348</v>
+      </c>
+      <c r="B9" s="42" t="n">
         <f aca="false">B4*0.9</f>
         <v>0</v>
       </c>
-      <c r="C9" s="36" t="n">
+      <c r="C9" s="42" t="n">
         <f aca="false">B4*1.1</f>
         <v>0</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>334</v>
-      </c>
-      <c r="E9" s="37" t="str">
+        <v>349</v>
+      </c>
+      <c r="E9" s="43" t="str">
         <f aca="false">IF(AND(B5&gt;=B9,B5&lt;C9),"◄ CURRENT","")</f>
         <v/>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>335</v>
-      </c>
-      <c r="B10" s="36" t="n">
+        <v>350</v>
+      </c>
+      <c r="B10" s="42" t="n">
         <f aca="false">B4*1.1</f>
         <v>0</v>
       </c>
-      <c r="C10" s="36" t="n">
+      <c r="C10" s="42" t="n">
         <f aca="false">B4*1.3</f>
         <v>0</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>336</v>
-      </c>
-      <c r="E10" s="37" t="str">
+        <v>351</v>
+      </c>
+      <c r="E10" s="43" t="str">
         <f aca="false">IF(AND(B5&gt;=B10,B5&lt;C10),"◄ CURRENT","")</f>
         <v/>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>337</v>
-      </c>
-      <c r="B11" s="36" t="n">
+        <v>352</v>
+      </c>
+      <c r="B11" s="42" t="n">
         <f aca="false">B4*1.3</f>
         <v>0</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>338</v>
+        <v>353</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>339</v>
-      </c>
-      <c r="E11" s="37" t="str">
+        <v>354</v>
+      </c>
+      <c r="E11" s="43" t="str">
         <f aca="false">IF(B5&gt;=B11,"◄ CURRENT","")</f>
         <v>◄ CURRENT</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="6" t="s">
-        <v>340</v>
+        <v>355</v>
       </c>
       <c r="B15" s="6"/>
       <c r="C15" s="6"/>
@@ -4021,79 +4256,79 @@
       <c r="E15" s="6"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="32" t="s">
-        <v>302</v>
-      </c>
-      <c r="B16" s="34"/>
+      <c r="A16" s="38" t="s">
+        <v>317</v>
+      </c>
+      <c r="B16" s="40"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="32" t="s">
-        <v>341</v>
-      </c>
-      <c r="B17" s="33"/>
+      <c r="A17" s="38" t="s">
+        <v>356</v>
+      </c>
+      <c r="B17" s="39"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
-        <v>329</v>
-      </c>
-      <c r="B19" s="36" t="n">
+        <v>344</v>
+      </c>
+      <c r="B19" s="42" t="n">
         <f aca="false">B16*0.6*B17</f>
         <v>0</v>
       </c>
-      <c r="C19" s="36" t="n">
+      <c r="C19" s="42" t="n">
         <f aca="false">B16*0.8*B17</f>
         <v>0</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="17" t="s">
-        <v>331</v>
-      </c>
-      <c r="B20" s="36" t="n">
+        <v>346</v>
+      </c>
+      <c r="B20" s="42" t="n">
         <f aca="false">B16*0.8*B17</f>
         <v>0</v>
       </c>
-      <c r="C20" s="36" t="n">
+      <c r="C20" s="42" t="n">
         <f aca="false">B16*1*B17</f>
         <v>0</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="s">
-        <v>333</v>
-      </c>
-      <c r="B21" s="36" t="n">
+        <v>348</v>
+      </c>
+      <c r="B21" s="42" t="n">
         <f aca="false">B16*1*B17</f>
         <v>0</v>
       </c>
-      <c r="C21" s="36" t="n">
+      <c r="C21" s="42" t="n">
         <f aca="false">B16*1.2*B17</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="17" t="s">
-        <v>335</v>
-      </c>
-      <c r="B22" s="36" t="n">
+        <v>350</v>
+      </c>
+      <c r="B22" s="42" t="n">
         <f aca="false">B16*1.2*B17</f>
         <v>0</v>
       </c>
-      <c r="C22" s="36" t="n">
+      <c r="C22" s="42" t="n">
         <f aca="false">B16*1.5*B17</f>
         <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="17" t="s">
-        <v>337</v>
-      </c>
-      <c r="B23" s="36" t="n">
+        <v>352</v>
+      </c>
+      <c r="B23" s="42" t="n">
         <f aca="false">B16*1.5*B17</f>
         <v>0</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>338</v>
+        <v>353</v>
       </c>
     </row>
   </sheetData>
@@ -4125,36 +4360,36 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>342</v>
+        <v>357</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>343</v>
+        <v>358</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>344</v>
+        <v>359</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>345</v>
+        <v>360</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
         <v>201</v>
       </c>
-      <c r="B4" s="35" t="n">
+      <c r="B4" s="41" t="n">
         <f aca="false">'1. Inputs'!B4</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>346</v>
-      </c>
-      <c r="B5" s="34"/>
+        <v>361</v>
+      </c>
+      <c r="B5" s="40"/>
       <c r="C5" s="12" t="str">
         <f aca="false">IF(B4=0,"-",(B5-B4)/B4)</f>
         <v>-</v>
@@ -4162,9 +4397,9 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>347</v>
-      </c>
-      <c r="B6" s="34"/>
+        <v>362</v>
+      </c>
+      <c r="B6" s="40"/>
       <c r="C6" s="12" t="str">
         <f aca="false">IF(B4=0,"-",(B6-B4)/B4)</f>
         <v>-</v>
@@ -4172,9 +4407,9 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>348</v>
-      </c>
-      <c r="B7" s="34"/>
+        <v>363</v>
+      </c>
+      <c r="B7" s="40"/>
       <c r="C7" s="12" t="str">
         <f aca="false">IF(B4=0,"-",(B7-B4)/B4)</f>
         <v>-</v>
@@ -4182,9 +4417,9 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>349</v>
-      </c>
-      <c r="B8" s="34"/>
+        <v>364</v>
+      </c>
+      <c r="B8" s="40"/>
       <c r="C8" s="12" t="str">
         <f aca="false">IF(B4=0,"-",(B8-B4)/B4)</f>
         <v>-</v>
@@ -4192,20 +4427,20 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>350</v>
+        <v>365</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>344</v>
+        <v>359</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>351</v>
+        <v>366</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>352</v>
-      </c>
-      <c r="B11" s="34"/>
+        <v>367</v>
+      </c>
+      <c r="B11" s="40"/>
       <c r="C11" s="12" t="str">
         <f aca="false">IF(B4=0,"-",(B11-B4)/B4)</f>
         <v>-</v>
@@ -4213,9 +4448,9 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>353</v>
-      </c>
-      <c r="B12" s="34"/>
+        <v>368</v>
+      </c>
+      <c r="B12" s="40"/>
       <c r="C12" s="12" t="str">
         <f aca="false">IF(B4=0,"-",(B12-B4)/B4)</f>
         <v>-</v>
@@ -4223,9 +4458,9 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>354</v>
-      </c>
-      <c r="B13" s="34"/>
+        <v>369</v>
+      </c>
+      <c r="B13" s="40"/>
       <c r="C13" s="12" t="str">
         <f aca="false">IF(B4=0,"-",(B13-B4)/B4)</f>
         <v>-</v>
@@ -4233,63 +4468,63 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="s">
-        <v>355</v>
-      </c>
-      <c r="B14" s="34"/>
+        <v>370</v>
+      </c>
+      <c r="B14" s="40"/>
       <c r="C14" s="12" t="str">
         <f aca="false">IF(B4=0,"-",(B14-B4)/B4)</f>
         <v>-</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="38" t="s">
-        <v>356</v>
+      <c r="A16" s="44" t="s">
+        <v>371</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="32" t="s">
-        <v>357</v>
+      <c r="A17" s="38" t="s">
+        <v>372</v>
       </c>
       <c r="B17" s="21"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="32" t="s">
-        <v>358</v>
+      <c r="A18" s="38" t="s">
+        <v>373</v>
       </c>
       <c r="B18" s="21"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="26" t="s">
-        <v>359</v>
-      </c>
-      <c r="B19" s="39" t="str">
+        <v>374</v>
+      </c>
+      <c r="B19" s="45" t="str">
         <f aca="false">IF(ABS(B17)=0,"-",ABS(B18)/ABS(B17))</f>
         <v>-</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>360</v>
+        <v>375</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>361</v>
+        <v>376</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>362</v>
+        <v>377</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>363</v>
+        <v>378</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>364</v>
+        <v>379</v>
       </c>
     </row>
   </sheetData>
@@ -4321,7 +4556,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>365</v>
+        <v>380</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -4330,7 +4565,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>366</v>
+        <v>381</v>
       </c>
       <c r="B3" s="6" t="s">
         <v>240</v>
@@ -4344,7 +4579,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="9" t="s">
-        <v>302</v>
+        <v>317</v>
       </c>
       <c r="B4" s="5"/>
       <c r="C4" s="5"/>
@@ -4380,7 +4615,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="9" t="s">
-        <v>367</v>
+        <v>382</v>
       </c>
       <c r="B7" s="12" t="n">
         <f aca="false">B5/100*B6/100</f>
@@ -4397,7 +4632,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>368</v>
+        <v>383</v>
       </c>
       <c r="B8" s="5" t="n">
         <v>1.5</v>
@@ -4413,81 +4648,81 @@
       <c r="A9" s="9" t="s">
         <v>201</v>
       </c>
-      <c r="B9" s="40" t="n">
+      <c r="B9" s="46" t="n">
         <f aca="false">'1. Inputs'!B4</f>
         <v>0</v>
       </c>
-      <c r="C9" s="40" t="n">
+      <c r="C9" s="46" t="n">
         <f aca="false">'1. Inputs'!B4</f>
         <v>0</v>
       </c>
-      <c r="D9" s="40" t="n">
+      <c r="D9" s="46" t="n">
         <f aca="false">'1. Inputs'!B4</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>369</v>
+        <v>384</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>370</v>
+        <v>385</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>306</v>
+        <v>321</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>307</v>
+        <v>322</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>308</v>
+        <v>323</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>309</v>
-      </c>
-      <c r="B12" s="31" t="n">
+        <v>324</v>
+      </c>
+      <c r="B12" s="37" t="n">
         <f aca="false">B4*(1+B7)^3</f>
         <v>0</v>
       </c>
-      <c r="C12" s="31" t="n">
+      <c r="C12" s="37" t="n">
         <f aca="false">B4*(1+B7)^5</f>
         <v>0</v>
       </c>
-      <c r="D12" s="31" t="n">
+      <c r="D12" s="37" t="n">
         <f aca="false">B4*(1+B7)^7</f>
         <v>0</v>
       </c>
-      <c r="E12" s="31" t="n">
+      <c r="E12" s="37" t="n">
         <f aca="false">B4*(1+B7)^10</f>
         <v>0</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>371</v>
-      </c>
-      <c r="B13" s="31" t="n">
+        <v>386</v>
+      </c>
+      <c r="B13" s="37" t="n">
         <f aca="false">B12*B8</f>
         <v>0</v>
       </c>
-      <c r="C13" s="31" t="n">
+      <c r="C13" s="37" t="n">
         <f aca="false">C12*B8</f>
         <v>0</v>
       </c>
-      <c r="D13" s="31" t="n">
+      <c r="D13" s="37" t="n">
         <f aca="false">D12*B8</f>
         <v>0</v>
       </c>
-      <c r="E13" s="31" t="n">
+      <c r="E13" s="37" t="n">
         <f aca="false">E12*B8</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="s">
-        <v>372</v>
+        <v>387</v>
       </c>
       <c r="B14" s="12" t="str">
         <f aca="false">IFERROR((B13/B9)^(1/3)-1,"-")</f>
@@ -4508,66 +4743,66 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="6" t="s">
-        <v>373</v>
+        <v>388</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>370</v>
+        <v>385</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>306</v>
+        <v>321</v>
       </c>
       <c r="D21" s="6" t="s">
-        <v>307</v>
+        <v>322</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>308</v>
+        <v>323</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="17" t="s">
-        <v>309</v>
-      </c>
-      <c r="B22" s="31" t="n">
+        <v>324</v>
+      </c>
+      <c r="B22" s="37" t="n">
         <f aca="false">C4*(1+C7)^3</f>
         <v>0</v>
       </c>
-      <c r="C22" s="31" t="n">
+      <c r="C22" s="37" t="n">
         <f aca="false">C4*(1+C7)^5</f>
         <v>0</v>
       </c>
-      <c r="D22" s="31" t="n">
+      <c r="D22" s="37" t="n">
         <f aca="false">C4*(1+C7)^7</f>
         <v>0</v>
       </c>
-      <c r="E22" s="31" t="n">
+      <c r="E22" s="37" t="n">
         <f aca="false">C4*(1+C7)^10</f>
         <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="17" t="s">
-        <v>371</v>
-      </c>
-      <c r="B23" s="31" t="n">
+        <v>386</v>
+      </c>
+      <c r="B23" s="37" t="n">
         <f aca="false">B22*C8</f>
         <v>0</v>
       </c>
-      <c r="C23" s="31" t="n">
+      <c r="C23" s="37" t="n">
         <f aca="false">C22*C8</f>
         <v>0</v>
       </c>
-      <c r="D23" s="31" t="n">
+      <c r="D23" s="37" t="n">
         <f aca="false">D22*C8</f>
         <v>0</v>
       </c>
-      <c r="E23" s="31" t="n">
+      <c r="E23" s="37" t="n">
         <f aca="false">E22*C8</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="17" t="s">
-        <v>372</v>
+        <v>387</v>
       </c>
       <c r="B24" s="12" t="str">
         <f aca="false">IFERROR((B23/C9)^(1/3)-1,"-")</f>
@@ -4588,66 +4823,66 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="6" t="s">
-        <v>374</v>
+        <v>389</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>370</v>
+        <v>385</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>306</v>
+        <v>321</v>
       </c>
       <c r="D31" s="6" t="s">
-        <v>307</v>
+        <v>322</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>308</v>
+        <v>323</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="17" t="s">
-        <v>309</v>
-      </c>
-      <c r="B32" s="31" t="n">
+        <v>324</v>
+      </c>
+      <c r="B32" s="37" t="n">
         <f aca="false">D4*(1+D7)^3</f>
         <v>0</v>
       </c>
-      <c r="C32" s="31" t="n">
+      <c r="C32" s="37" t="n">
         <f aca="false">D4*(1+D7)^5</f>
         <v>0</v>
       </c>
-      <c r="D32" s="31" t="n">
+      <c r="D32" s="37" t="n">
         <f aca="false">D4*(1+D7)^7</f>
         <v>0</v>
       </c>
-      <c r="E32" s="31" t="n">
+      <c r="E32" s="37" t="n">
         <f aca="false">D4*(1+D7)^10</f>
         <v>0</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="17" t="s">
-        <v>371</v>
-      </c>
-      <c r="B33" s="31" t="n">
+        <v>386</v>
+      </c>
+      <c r="B33" s="37" t="n">
         <f aca="false">B32*D8</f>
         <v>0</v>
       </c>
-      <c r="C33" s="31" t="n">
+      <c r="C33" s="37" t="n">
         <f aca="false">C32*D8</f>
         <v>0</v>
       </c>
-      <c r="D33" s="31" t="n">
+      <c r="D33" s="37" t="n">
         <f aca="false">D32*D8</f>
         <v>0</v>
       </c>
-      <c r="E33" s="31" t="n">
+      <c r="E33" s="37" t="n">
         <f aca="false">E32*D8</f>
         <v>0</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="17" t="s">
-        <v>372</v>
+        <v>387</v>
       </c>
       <c r="B34" s="12" t="str">
         <f aca="false">IFERROR((B33/D9)^(1/3)-1,"-")</f>
@@ -4695,7 +4930,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>375</v>
+        <v>390</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -4711,13 +4946,13 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>376</v>
+        <v>391</v>
       </c>
       <c r="B3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>302</v>
+        <v>317</v>
       </c>
       <c r="B4" s="5"/>
     </row>
@@ -4731,7 +4966,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>377</v>
+        <v>392</v>
       </c>
       <c r="B6" s="5" t="n">
         <v>11</v>
@@ -4747,7 +4982,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>367</v>
+        <v>382</v>
       </c>
       <c r="B8" s="12" t="n">
         <f aca="false">B5/100*B7/100</f>
@@ -4756,7 +4991,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>378</v>
+        <v>393</v>
       </c>
       <c r="B9" s="12" t="n">
         <f aca="false">(B5-B6)/100</f>
@@ -4765,7 +5000,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>379</v>
+        <v>394</v>
       </c>
       <c r="B10" s="5" t="n">
         <v>4</v>
@@ -4791,7 +5026,7 @@
     </row>
     <row r="14" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="6" t="s">
-        <v>380</v>
+        <v>395</v>
       </c>
       <c r="B14" s="6"/>
       <c r="C14" s="6"/>
@@ -4898,7 +5133,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="17" t="s">
-        <v>381</v>
+        <v>396</v>
       </c>
       <c r="C17" s="11" t="n">
         <f aca="false">B16*B9</f>
@@ -4996,7 +5231,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="17" t="s">
-        <v>382</v>
+        <v>397</v>
       </c>
       <c r="C19" s="11" t="n">
         <f aca="false">C17*C18</f>
@@ -5045,36 +5280,36 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="17" t="s">
-        <v>302</v>
-      </c>
-      <c r="B21" s="31" t="n">
+        <v>317</v>
+      </c>
+      <c r="B21" s="37" t="n">
         <f aca="false">B4</f>
         <v>0</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="17" t="s">
-        <v>383</v>
-      </c>
-      <c r="B22" s="31" t="n">
+        <v>398</v>
+      </c>
+      <c r="B22" s="37" t="n">
         <f aca="false">SUM(C19:L19)</f>
         <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="17" t="s">
-        <v>384</v>
-      </c>
-      <c r="B23" s="31" t="n">
+        <v>399</v>
+      </c>
+      <c r="B23" s="37" t="n">
         <f aca="false">M19</f>
         <v>0</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="38" t="s">
-        <v>385</v>
-      </c>
-      <c r="B24" s="41" t="n">
+      <c r="A24" s="44" t="s">
+        <v>400</v>
+      </c>
+      <c r="B24" s="47" t="n">
         <f aca="false">B21+B22+B23</f>
         <v>0</v>
       </c>
@@ -5126,7 +5361,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>386</v>
+        <v>401</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -5141,19 +5376,19 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>387</v>
+        <v>402</v>
       </c>
       <c r="B3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="32" t="s">
-        <v>388</v>
+      <c r="A4" s="38" t="s">
+        <v>403</v>
       </c>
       <c r="B4" s="5" t="n">
         <v>70</v>
       </c>
-      <c r="C4" s="42" t="s">
-        <v>389</v>
+      <c r="C4" s="48" t="s">
+        <v>404</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5256,7 +5491,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="9" t="s">
-        <v>390</v>
+        <v>405</v>
       </c>
       <c r="B8" s="11" t="n">
         <f aca="false">'1. Inputs'!B14</f>
@@ -5305,7 +5540,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="9" t="s">
-        <v>391</v>
+        <v>406</v>
       </c>
       <c r="B9" s="11" t="n">
         <f aca="false">'1. Inputs'!B14*$B$4/100</f>
@@ -5354,7 +5589,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="9" t="s">
-        <v>392</v>
+        <v>407</v>
       </c>
       <c r="B10" s="11" t="n">
         <f aca="false">'1. Inputs'!B18+'1. Inputs'!B14-'1. Inputs'!B14*$B$4/100</f>
@@ -5403,7 +5638,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>393</v>
+        <v>408</v>
       </c>
       <c r="B11" s="11" t="str">
         <f aca="false">IF('1. Inputs'!$B$5=0,"-",B10/'1. Inputs'!$B$5)</f>
@@ -5452,7 +5687,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>394</v>
+        <v>409</v>
       </c>
       <c r="B12" s="12" t="s">
         <v>124</v>
@@ -5500,104 +5735,104 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>395</v>
-      </c>
-      <c r="B13" s="19" t="e">
-        <f aca="false">IF(B11=0,"-",'1. Inputs'!$B$4/B11)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C13" s="19" t="e">
-        <f aca="false">IF(C11=0,"-",'1. Inputs'!$B$4/C11)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D13" s="19" t="e">
-        <f aca="false">IF(D11=0,"-",'1. Inputs'!$B$4/D11)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E13" s="19" t="e">
-        <f aca="false">IF(E11=0,"-",'1. Inputs'!$B$4/E11)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F13" s="19" t="e">
-        <f aca="false">IF(F11=0,"-",'1. Inputs'!$B$4/F11)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G13" s="19" t="e">
-        <f aca="false">IF(G11=0,"-",'1. Inputs'!$B$4/G11)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="H13" s="19" t="e">
-        <f aca="false">IF(H11=0,"-",'1. Inputs'!$B$4/H11)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I13" s="19" t="e">
-        <f aca="false">IF(I11=0,"-",'1. Inputs'!$B$4/I11)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="J13" s="19" t="e">
-        <f aca="false">IF(J11=0,"-",'1. Inputs'!$B$4/J11)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K13" s="19" t="e">
-        <f aca="false">IF(K11=0,"-",'1. Inputs'!$B$4/K11)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L13" s="19" t="e">
-        <f aca="false">IF(L11=0,"-",'1. Inputs'!$B$4/L11)</f>
-        <v>#VALUE!</v>
+        <v>410</v>
+      </c>
+      <c r="B13" s="19" t="str">
+        <f aca="false">IFERROR('1. Inputs'!$B$4/B11,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="C13" s="19" t="str">
+        <f aca="false">IFERROR('1. Inputs'!$B$4/C11,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="D13" s="19" t="str">
+        <f aca="false">IFERROR('1. Inputs'!$B$4/D11,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="E13" s="19" t="str">
+        <f aca="false">IFERROR('1. Inputs'!$B$4/E11,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="F13" s="19" t="str">
+        <f aca="false">IFERROR('1. Inputs'!$B$4/F11,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="G13" s="19" t="str">
+        <f aca="false">IFERROR('1. Inputs'!$B$4/G11,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="H13" s="19" t="str">
+        <f aca="false">IFERROR('1. Inputs'!$B$4/H11,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="I13" s="19" t="str">
+        <f aca="false">IFERROR('1. Inputs'!$B$4/I11,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="J13" s="19" t="str">
+        <f aca="false">IFERROR('1. Inputs'!$B$4/J11,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="K13" s="19" t="str">
+        <f aca="false">IFERROR('1. Inputs'!$B$4/K11,"-")</f>
+        <v>-</v>
+      </c>
+      <c r="L13" s="19" t="str">
+        <f aca="false">IFERROR('1. Inputs'!$B$4/L11,"-")</f>
+        <v>-</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>396</v>
+        <v>411</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>397</v>
+        <v>412</v>
       </c>
       <c r="B15" s="11" t="n">
-        <f aca="false">'1. Inputs'!B54</f>
+        <f aca="false">'1. Inputs'!B55</f>
         <v>0</v>
       </c>
       <c r="C15" s="11" t="n">
-        <f aca="false">'1. Inputs'!C54</f>
+        <f aca="false">'1. Inputs'!C55</f>
         <v>0</v>
       </c>
       <c r="D15" s="11" t="n">
-        <f aca="false">'1. Inputs'!D54</f>
+        <f aca="false">'1. Inputs'!D55</f>
         <v>0</v>
       </c>
       <c r="E15" s="11" t="n">
-        <f aca="false">'1. Inputs'!E54</f>
+        <f aca="false">'1. Inputs'!E55</f>
         <v>0</v>
       </c>
       <c r="F15" s="11" t="n">
-        <f aca="false">'1. Inputs'!F54</f>
+        <f aca="false">'1. Inputs'!F55</f>
         <v>0</v>
       </c>
       <c r="G15" s="11" t="n">
-        <f aca="false">'1. Inputs'!G54</f>
+        <f aca="false">'1. Inputs'!G55</f>
         <v>0</v>
       </c>
       <c r="H15" s="11" t="n">
-        <f aca="false">'1. Inputs'!H54</f>
+        <f aca="false">'1. Inputs'!H55</f>
         <v>0</v>
       </c>
       <c r="I15" s="11" t="n">
-        <f aca="false">'1. Inputs'!I54</f>
+        <f aca="false">'1. Inputs'!I55</f>
         <v>0</v>
       </c>
       <c r="J15" s="11" t="n">
-        <f aca="false">'1. Inputs'!J54</f>
+        <f aca="false">'1. Inputs'!J55</f>
         <v>0</v>
       </c>
       <c r="K15" s="11" t="n">
-        <f aca="false">'1. Inputs'!K54</f>
+        <f aca="false">'1. Inputs'!K55</f>
         <v>0</v>
       </c>
       <c r="L15" s="11" t="n">
-        <f aca="false">'1. Inputs'!L54</f>
+        <f aca="false">'1. Inputs'!L55</f>
         <v>0</v>
       </c>
     </row>
@@ -5606,47 +5841,47 @@
         <v>179</v>
       </c>
       <c r="B16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!B12=0),"-",ABS('1. Inputs'!B54)/'1. Inputs'!B12)</f>
+        <f aca="false">IF(OR('1. Inputs'!B12=0),"-",ABS('1. Inputs'!B55)/'1. Inputs'!B12)</f>
         <v>-</v>
       </c>
       <c r="C16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!C12=0),"-",ABS('1. Inputs'!C54)/'1. Inputs'!C12)</f>
+        <f aca="false">IF(OR('1. Inputs'!C12=0),"-",ABS('1. Inputs'!C55)/'1. Inputs'!C12)</f>
         <v>-</v>
       </c>
       <c r="D16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!D12=0),"-",ABS('1. Inputs'!D54)/'1. Inputs'!D12)</f>
+        <f aca="false">IF(OR('1. Inputs'!D12=0),"-",ABS('1. Inputs'!D55)/'1. Inputs'!D12)</f>
         <v>-</v>
       </c>
       <c r="E16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!E12=0),"-",ABS('1. Inputs'!E54)/'1. Inputs'!E12)</f>
+        <f aca="false">IF(OR('1. Inputs'!E12=0),"-",ABS('1. Inputs'!E55)/'1. Inputs'!E12)</f>
         <v>-</v>
       </c>
       <c r="F16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!F12=0),"-",ABS('1. Inputs'!F54)/'1. Inputs'!F12)</f>
+        <f aca="false">IF(OR('1. Inputs'!F12=0),"-",ABS('1. Inputs'!F55)/'1. Inputs'!F12)</f>
         <v>-</v>
       </c>
       <c r="G16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!G12=0),"-",ABS('1. Inputs'!G54)/'1. Inputs'!G12)</f>
+        <f aca="false">IF(OR('1. Inputs'!G12=0),"-",ABS('1. Inputs'!G55)/'1. Inputs'!G12)</f>
         <v>-</v>
       </c>
       <c r="H16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!H12=0),"-",ABS('1. Inputs'!H54)/'1. Inputs'!H12)</f>
+        <f aca="false">IF(OR('1. Inputs'!H12=0),"-",ABS('1. Inputs'!H55)/'1. Inputs'!H12)</f>
         <v>-</v>
       </c>
       <c r="I16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!I12=0),"-",ABS('1. Inputs'!I54)/'1. Inputs'!I12)</f>
+        <f aca="false">IF(OR('1. Inputs'!I12=0),"-",ABS('1. Inputs'!I55)/'1. Inputs'!I12)</f>
         <v>-</v>
       </c>
       <c r="J16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!J12=0),"-",ABS('1. Inputs'!J54)/'1. Inputs'!J12)</f>
+        <f aca="false">IF(OR('1. Inputs'!J12=0),"-",ABS('1. Inputs'!J55)/'1. Inputs'!J12)</f>
         <v>-</v>
       </c>
       <c r="K16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!K12=0),"-",ABS('1. Inputs'!K54)/'1. Inputs'!K12)</f>
+        <f aca="false">IF(OR('1. Inputs'!K12=0),"-",ABS('1. Inputs'!K55)/'1. Inputs'!K12)</f>
         <v>-</v>
       </c>
       <c r="L16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!L12=0),"-",ABS('1. Inputs'!L54)/'1. Inputs'!L12)</f>
+        <f aca="false">IF(OR('1. Inputs'!L12=0),"-",ABS('1. Inputs'!L55)/'1. Inputs'!L12)</f>
         <v>-</v>
       </c>
     </row>
@@ -5655,96 +5890,96 @@
         <v>157</v>
       </c>
       <c r="B17" s="11" t="n">
-        <f aca="false">'1. Inputs'!B57</f>
+        <f aca="false">'1. Inputs'!B58</f>
         <v>0</v>
       </c>
       <c r="C17" s="11" t="n">
-        <f aca="false">'1. Inputs'!C57</f>
+        <f aca="false">'1. Inputs'!C58</f>
         <v>0</v>
       </c>
       <c r="D17" s="11" t="n">
-        <f aca="false">'1. Inputs'!D57</f>
+        <f aca="false">'1. Inputs'!D58</f>
         <v>0</v>
       </c>
       <c r="E17" s="11" t="n">
-        <f aca="false">'1. Inputs'!E57</f>
+        <f aca="false">'1. Inputs'!E58</f>
         <v>0</v>
       </c>
       <c r="F17" s="11" t="n">
-        <f aca="false">'1. Inputs'!F57</f>
+        <f aca="false">'1. Inputs'!F58</f>
         <v>0</v>
       </c>
       <c r="G17" s="11" t="n">
-        <f aca="false">'1. Inputs'!G57</f>
+        <f aca="false">'1. Inputs'!G58</f>
         <v>0</v>
       </c>
       <c r="H17" s="11" t="n">
-        <f aca="false">'1. Inputs'!H57</f>
+        <f aca="false">'1. Inputs'!H58</f>
         <v>0</v>
       </c>
       <c r="I17" s="11" t="n">
-        <f aca="false">'1. Inputs'!I57</f>
+        <f aca="false">'1. Inputs'!I58</f>
         <v>0</v>
       </c>
       <c r="J17" s="11" t="n">
-        <f aca="false">'1. Inputs'!J57</f>
+        <f aca="false">'1. Inputs'!J58</f>
         <v>0</v>
       </c>
       <c r="K17" s="11" t="n">
-        <f aca="false">'1. Inputs'!K57</f>
+        <f aca="false">'1. Inputs'!K58</f>
         <v>0</v>
       </c>
       <c r="L17" s="11" t="n">
-        <f aca="false">'1. Inputs'!L57</f>
+        <f aca="false">'1. Inputs'!L58</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="9" t="s">
-        <v>398</v>
+        <v>413</v>
       </c>
       <c r="B18" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!B12=0),"-",'1. Inputs'!B57/'1. Inputs'!B12)</f>
+        <f aca="false">IF(OR('1. Inputs'!B12=0),"-",'1. Inputs'!B58/'1. Inputs'!B12)</f>
         <v>-</v>
       </c>
       <c r="C18" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!C12=0),"-",'1. Inputs'!C57/'1. Inputs'!C12)</f>
+        <f aca="false">IF(OR('1. Inputs'!C12=0),"-",'1. Inputs'!C58/'1. Inputs'!C12)</f>
         <v>-</v>
       </c>
       <c r="D18" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!D12=0),"-",'1. Inputs'!D57/'1. Inputs'!D12)</f>
+        <f aca="false">IF(OR('1. Inputs'!D12=0),"-",'1. Inputs'!D58/'1. Inputs'!D12)</f>
         <v>-</v>
       </c>
       <c r="E18" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!E12=0),"-",'1. Inputs'!E57/'1. Inputs'!E12)</f>
+        <f aca="false">IF(OR('1. Inputs'!E12=0),"-",'1. Inputs'!E58/'1. Inputs'!E12)</f>
         <v>-</v>
       </c>
       <c r="F18" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!F12=0),"-",'1. Inputs'!F57/'1. Inputs'!F12)</f>
+        <f aca="false">IF(OR('1. Inputs'!F12=0),"-",'1. Inputs'!F58/'1. Inputs'!F12)</f>
         <v>-</v>
       </c>
       <c r="G18" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!G12=0),"-",'1. Inputs'!G57/'1. Inputs'!G12)</f>
+        <f aca="false">IF(OR('1. Inputs'!G12=0),"-",'1. Inputs'!G58/'1. Inputs'!G12)</f>
         <v>-</v>
       </c>
       <c r="H18" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!H12=0),"-",'1. Inputs'!H57/'1. Inputs'!H12)</f>
+        <f aca="false">IF(OR('1. Inputs'!H12=0),"-",'1. Inputs'!H58/'1. Inputs'!H12)</f>
         <v>-</v>
       </c>
       <c r="I18" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!I12=0),"-",'1. Inputs'!I57/'1. Inputs'!I12)</f>
+        <f aca="false">IF(OR('1. Inputs'!I12=0),"-",'1. Inputs'!I58/'1. Inputs'!I12)</f>
         <v>-</v>
       </c>
       <c r="J18" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!J12=0),"-",'1. Inputs'!J57/'1. Inputs'!J12)</f>
+        <f aca="false">IF(OR('1. Inputs'!J12=0),"-",'1. Inputs'!J58/'1. Inputs'!J12)</f>
         <v>-</v>
       </c>
       <c r="K18" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!K12=0),"-",'1. Inputs'!K57/'1. Inputs'!K12)</f>
+        <f aca="false">IF(OR('1. Inputs'!K12=0),"-",'1. Inputs'!K58/'1. Inputs'!K12)</f>
         <v>-</v>
       </c>
       <c r="L18" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!L12=0),"-",'1. Inputs'!L57/'1. Inputs'!L12)</f>
+        <f aca="false">IF(OR('1. Inputs'!L12=0),"-",'1. Inputs'!L58/'1. Inputs'!L12)</f>
         <v>-</v>
       </c>
     </row>
@@ -5753,47 +5988,47 @@
         <v>158</v>
       </c>
       <c r="B19" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!B18=0),"-",'1. Inputs'!B57/'1. Inputs'!B18)</f>
+        <f aca="false">IF(OR('1. Inputs'!B18=0),"-",'1. Inputs'!B58/'1. Inputs'!B18)</f>
         <v>-</v>
       </c>
       <c r="C19" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!C18=0),"-",'1. Inputs'!C57/'1. Inputs'!C18)</f>
+        <f aca="false">IF(OR('1. Inputs'!C18=0),"-",'1. Inputs'!C58/'1. Inputs'!C18)</f>
         <v>-</v>
       </c>
       <c r="D19" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!D18=0),"-",'1. Inputs'!D57/'1. Inputs'!D18)</f>
+        <f aca="false">IF(OR('1. Inputs'!D18=0),"-",'1. Inputs'!D58/'1. Inputs'!D18)</f>
         <v>-</v>
       </c>
       <c r="E19" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!E18=0),"-",'1. Inputs'!E57/'1. Inputs'!E18)</f>
+        <f aca="false">IF(OR('1. Inputs'!E18=0),"-",'1. Inputs'!E58/'1. Inputs'!E18)</f>
         <v>-</v>
       </c>
       <c r="F19" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!F18=0),"-",'1. Inputs'!F57/'1. Inputs'!F18)</f>
+        <f aca="false">IF(OR('1. Inputs'!F18=0),"-",'1. Inputs'!F58/'1. Inputs'!F18)</f>
         <v>-</v>
       </c>
       <c r="G19" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!G18=0),"-",'1. Inputs'!G57/'1. Inputs'!G18)</f>
+        <f aca="false">IF(OR('1. Inputs'!G18=0),"-",'1. Inputs'!G58/'1. Inputs'!G18)</f>
         <v>-</v>
       </c>
       <c r="H19" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!H18=0),"-",'1. Inputs'!H57/'1. Inputs'!H18)</f>
+        <f aca="false">IF(OR('1. Inputs'!H18=0),"-",'1. Inputs'!H58/'1. Inputs'!H18)</f>
         <v>-</v>
       </c>
       <c r="I19" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!I18=0),"-",'1. Inputs'!I57/'1. Inputs'!I18)</f>
+        <f aca="false">IF(OR('1. Inputs'!I18=0),"-",'1. Inputs'!I58/'1. Inputs'!I18)</f>
         <v>-</v>
       </c>
       <c r="J19" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!J18=0),"-",'1. Inputs'!J57/'1. Inputs'!J18)</f>
+        <f aca="false">IF(OR('1. Inputs'!J18=0),"-",'1. Inputs'!J58/'1. Inputs'!J18)</f>
         <v>-</v>
       </c>
       <c r="K19" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!K18=0),"-",'1. Inputs'!K57/'1. Inputs'!K18)</f>
+        <f aca="false">IF(OR('1. Inputs'!K18=0),"-",'1. Inputs'!K58/'1. Inputs'!K18)</f>
         <v>-</v>
       </c>
       <c r="L19" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!L18=0),"-",'1. Inputs'!L57/'1. Inputs'!L18)</f>
+        <f aca="false">IF(OR('1. Inputs'!L18=0),"-",'1. Inputs'!L58/'1. Inputs'!L18)</f>
         <v>-</v>
       </c>
     </row>
@@ -5827,118 +6062,118 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>399</v>
+        <v>414</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>400</v>
+        <v>415</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>401</v>
+        <v>416</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>402</v>
+        <v>417</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>403</v>
-      </c>
-      <c r="B4" s="43"/>
+        <v>418</v>
+      </c>
+      <c r="B4" s="49"/>
       <c r="C4" s="5"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>404</v>
-      </c>
-      <c r="B5" s="43"/>
+        <v>419</v>
+      </c>
+      <c r="B5" s="49"/>
       <c r="C5" s="5"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>405</v>
-      </c>
-      <c r="B6" s="43"/>
+        <v>420</v>
+      </c>
+      <c r="B6" s="49"/>
       <c r="C6" s="5"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>406</v>
-      </c>
-      <c r="B7" s="43"/>
+        <v>421</v>
+      </c>
+      <c r="B7" s="49"/>
       <c r="C7" s="5"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>407</v>
-      </c>
-      <c r="B8" s="43"/>
+        <v>422</v>
+      </c>
+      <c r="B8" s="49"/>
       <c r="C8" s="5"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>408</v>
-      </c>
-      <c r="B9" s="43"/>
+        <v>423</v>
+      </c>
+      <c r="B9" s="49"/>
       <c r="C9" s="5"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>409</v>
-      </c>
-      <c r="B10" s="43"/>
+        <v>424</v>
+      </c>
+      <c r="B10" s="49"/>
       <c r="C10" s="5"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>410</v>
-      </c>
-      <c r="B11" s="43"/>
+        <v>425</v>
+      </c>
+      <c r="B11" s="49"/>
       <c r="C11" s="5"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>411</v>
-      </c>
-      <c r="B12" s="43"/>
+        <v>426</v>
+      </c>
+      <c r="B12" s="49"/>
       <c r="C12" s="5"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>412</v>
-      </c>
-      <c r="B13" s="43"/>
+        <v>427</v>
+      </c>
+      <c r="B13" s="49"/>
       <c r="C13" s="5"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="38" t="s">
-        <v>413</v>
-      </c>
-      <c r="B15" s="44" t="e">
-        <f aca="false">AVERAGE(B4:B13)</f>
-        <v>#DIV/0!</v>
+      <c r="A15" s="44" t="s">
+        <v>428</v>
+      </c>
+      <c r="B15" s="50" t="str">
+        <f aca="false">IFERROR(AVERAGE(B4:B13),"-")</f>
+        <v>-</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="38" t="s">
-        <v>414</v>
-      </c>
-      <c r="B16" s="45" t="e">
-        <f aca="false">IF(B15&gt;=8,"STRONG BUY",IF(B15&gt;=6.5,"BUY",IF(B15&gt;=5,"HOLD",IF(B15&gt;=3.5,"AVOID","SELL"))))</f>
-        <v>#DIV/0!</v>
+      <c r="A16" s="44" t="s">
+        <v>429</v>
+      </c>
+      <c r="B16" s="51" t="str">
+        <f aca="false">IF(OR(B15="-",B15=0),"-",IF(B15&gt;=8,"STRONG BUY",IF(B15&gt;=6.5,"BUY",IF(B15&gt;=5,"HOLD",IF(B15&gt;=3.5,"AVOID","SELL")))))</f>
+        <v>-</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>415</v>
+        <v>430</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>416</v>
+        <v>431</v>
       </c>
     </row>
   </sheetData>
@@ -8023,49 +8258,49 @@
       <c r="A4" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="B4" s="11" t="str">
-        <f aca="false">'1. Inputs'!B31</f>
-        <v>FY1 (Oldest)</v>
-      </c>
-      <c r="C4" s="11" t="str">
-        <f aca="false">'1. Inputs'!C31</f>
-        <v>FY2</v>
-      </c>
-      <c r="D4" s="11" t="str">
-        <f aca="false">'1. Inputs'!D31</f>
-        <v>FY3</v>
-      </c>
-      <c r="E4" s="11" t="str">
-        <f aca="false">'1. Inputs'!E31</f>
-        <v>FY4</v>
-      </c>
-      <c r="F4" s="11" t="str">
-        <f aca="false">'1. Inputs'!F31</f>
-        <v>FY5</v>
-      </c>
-      <c r="G4" s="11" t="str">
-        <f aca="false">'1. Inputs'!G31</f>
-        <v>FY6</v>
-      </c>
-      <c r="H4" s="11" t="str">
-        <f aca="false">'1. Inputs'!H31</f>
-        <v>FY7</v>
-      </c>
-      <c r="I4" s="11" t="str">
-        <f aca="false">'1. Inputs'!I31</f>
-        <v>FY8</v>
-      </c>
-      <c r="J4" s="11" t="str">
-        <f aca="false">'1. Inputs'!J31</f>
-        <v>FY9</v>
-      </c>
-      <c r="K4" s="11" t="str">
-        <f aca="false">'1. Inputs'!K31</f>
-        <v>FY10 (Latest)</v>
-      </c>
-      <c r="L4" s="11" t="str">
-        <f aca="false">'1. Inputs'!L31</f>
-        <v>TTM</v>
+      <c r="B4" s="11" t="n">
+        <f aca="false">'1. Inputs'!B32</f>
+        <v>0</v>
+      </c>
+      <c r="C4" s="11" t="n">
+        <f aca="false">'1. Inputs'!C32</f>
+        <v>0</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <f aca="false">'1. Inputs'!D32</f>
+        <v>0</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <f aca="false">'1. Inputs'!E32</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <f aca="false">'1. Inputs'!F32</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="11" t="n">
+        <f aca="false">'1. Inputs'!G32</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <f aca="false">'1. Inputs'!H32</f>
+        <v>0</v>
+      </c>
+      <c r="I4" s="11" t="n">
+        <f aca="false">'1. Inputs'!I32</f>
+        <v>0</v>
+      </c>
+      <c r="J4" s="11" t="n">
+        <f aca="false">'1. Inputs'!J32</f>
+        <v>0</v>
+      </c>
+      <c r="K4" s="11" t="n">
+        <f aca="false">'1. Inputs'!K32</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="11" t="n">
+        <f aca="false">'1. Inputs'!L32</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8075,45 +8310,45 @@
       <c r="B5" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="C5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!B31=0,'1. Inputs'!B31=""),"-",('1. Inputs'!C31-'1. Inputs'!B31)/ABS('1. Inputs'!B31))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!C31=0,'1. Inputs'!C31=""),"-",('1. Inputs'!D31-'1. Inputs'!C31)/ABS('1. Inputs'!C31))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!D31=0,'1. Inputs'!D31=""),"-",('1. Inputs'!E31-'1. Inputs'!D31)/ABS('1. Inputs'!D31))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!E31=0,'1. Inputs'!E31=""),"-",('1. Inputs'!F31-'1. Inputs'!E31)/ABS('1. Inputs'!E31))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!F31=0,'1. Inputs'!F31=""),"-",('1. Inputs'!G31-'1. Inputs'!F31)/ABS('1. Inputs'!F31))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="H5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!G31=0,'1. Inputs'!G31=""),"-",('1. Inputs'!H31-'1. Inputs'!G31)/ABS('1. Inputs'!G31))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!H31=0,'1. Inputs'!H31=""),"-",('1. Inputs'!I31-'1. Inputs'!H31)/ABS('1. Inputs'!H31))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="J5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!I31=0,'1. Inputs'!I31=""),"-",('1. Inputs'!J31-'1. Inputs'!I31)/ABS('1. Inputs'!I31))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!J31=0,'1. Inputs'!J31=""),"-",('1. Inputs'!K31-'1. Inputs'!J31)/ABS('1. Inputs'!J31))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!K31=0,'1. Inputs'!K31=""),"-",('1. Inputs'!L31-'1. Inputs'!K31)/ABS('1. Inputs'!K31))</f>
-        <v>#VALUE!</v>
+      <c r="C5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!B32=0,'1. Inputs'!B32=""),"-",('1. Inputs'!C32-'1. Inputs'!B32)/ABS('1. Inputs'!B32))</f>
+        <v>-</v>
+      </c>
+      <c r="D5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!C32=0,'1. Inputs'!C32=""),"-",('1. Inputs'!D32-'1. Inputs'!C32)/ABS('1. Inputs'!C32))</f>
+        <v>-</v>
+      </c>
+      <c r="E5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!D32=0,'1. Inputs'!D32=""),"-",('1. Inputs'!E32-'1. Inputs'!D32)/ABS('1. Inputs'!D32))</f>
+        <v>-</v>
+      </c>
+      <c r="F5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!E32=0,'1. Inputs'!E32=""),"-",('1. Inputs'!F32-'1. Inputs'!E32)/ABS('1. Inputs'!E32))</f>
+        <v>-</v>
+      </c>
+      <c r="G5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!F32=0,'1. Inputs'!F32=""),"-",('1. Inputs'!G32-'1. Inputs'!F32)/ABS('1. Inputs'!F32))</f>
+        <v>-</v>
+      </c>
+      <c r="H5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!G32=0,'1. Inputs'!G32=""),"-",('1. Inputs'!H32-'1. Inputs'!G32)/ABS('1. Inputs'!G32))</f>
+        <v>-</v>
+      </c>
+      <c r="I5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!H32=0,'1. Inputs'!H32=""),"-",('1. Inputs'!I32-'1. Inputs'!H32)/ABS('1. Inputs'!H32))</f>
+        <v>-</v>
+      </c>
+      <c r="J5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!I32=0,'1. Inputs'!I32=""),"-",('1. Inputs'!J32-'1. Inputs'!I32)/ABS('1. Inputs'!I32))</f>
+        <v>-</v>
+      </c>
+      <c r="K5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!J32=0,'1. Inputs'!J32=""),"-",('1. Inputs'!K32-'1. Inputs'!J32)/ABS('1. Inputs'!J32))</f>
+        <v>-</v>
+      </c>
+      <c r="L5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!K32=0,'1. Inputs'!K32=""),"-",('1. Inputs'!L32-'1. Inputs'!K32)/ABS('1. Inputs'!K32))</f>
+        <v>-</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8121,47 +8356,47 @@
         <v>76</v>
       </c>
       <c r="B6" s="11" t="n">
-        <f aca="false">'1. Inputs'!B32</f>
+        <f aca="false">'1. Inputs'!B33</f>
         <v>0</v>
       </c>
       <c r="C6" s="11" t="n">
-        <f aca="false">'1. Inputs'!C32</f>
+        <f aca="false">'1. Inputs'!C33</f>
         <v>0</v>
       </c>
       <c r="D6" s="11" t="n">
-        <f aca="false">'1. Inputs'!D32</f>
+        <f aca="false">'1. Inputs'!D33</f>
         <v>0</v>
       </c>
       <c r="E6" s="11" t="n">
-        <f aca="false">'1. Inputs'!E32</f>
+        <f aca="false">'1. Inputs'!E33</f>
         <v>0</v>
       </c>
       <c r="F6" s="11" t="n">
-        <f aca="false">'1. Inputs'!F32</f>
+        <f aca="false">'1. Inputs'!F33</f>
         <v>0</v>
       </c>
       <c r="G6" s="11" t="n">
-        <f aca="false">'1. Inputs'!G32</f>
+        <f aca="false">'1. Inputs'!G33</f>
         <v>0</v>
       </c>
       <c r="H6" s="11" t="n">
-        <f aca="false">'1. Inputs'!H32</f>
+        <f aca="false">'1. Inputs'!H33</f>
         <v>0</v>
       </c>
       <c r="I6" s="11" t="n">
-        <f aca="false">'1. Inputs'!I32</f>
+        <f aca="false">'1. Inputs'!I33</f>
         <v>0</v>
       </c>
       <c r="J6" s="11" t="n">
-        <f aca="false">'1. Inputs'!J32</f>
+        <f aca="false">'1. Inputs'!J33</f>
         <v>0</v>
       </c>
       <c r="K6" s="11" t="n">
-        <f aca="false">'1. Inputs'!K32</f>
+        <f aca="false">'1. Inputs'!K33</f>
         <v>0</v>
       </c>
       <c r="L6" s="11" t="n">
-        <f aca="false">'1. Inputs'!L32</f>
+        <f aca="false">'1. Inputs'!L33</f>
         <v>0</v>
       </c>
     </row>
@@ -8170,47 +8405,47 @@
         <v>77</v>
       </c>
       <c r="B7" s="11" t="n">
-        <f aca="false">'1. Inputs'!B33</f>
+        <f aca="false">'1. Inputs'!B34</f>
         <v>0</v>
       </c>
       <c r="C7" s="11" t="n">
-        <f aca="false">'1. Inputs'!C33</f>
+        <f aca="false">'1. Inputs'!C34</f>
         <v>0</v>
       </c>
       <c r="D7" s="11" t="n">
-        <f aca="false">'1. Inputs'!D33</f>
+        <f aca="false">'1. Inputs'!D34</f>
         <v>0</v>
       </c>
       <c r="E7" s="11" t="n">
-        <f aca="false">'1. Inputs'!E33</f>
+        <f aca="false">'1. Inputs'!E34</f>
         <v>0</v>
       </c>
       <c r="F7" s="11" t="n">
-        <f aca="false">'1. Inputs'!F33</f>
+        <f aca="false">'1. Inputs'!F34</f>
         <v>0</v>
       </c>
       <c r="G7" s="11" t="n">
-        <f aca="false">'1. Inputs'!G33</f>
+        <f aca="false">'1. Inputs'!G34</f>
         <v>0</v>
       </c>
       <c r="H7" s="11" t="n">
-        <f aca="false">'1. Inputs'!H33</f>
+        <f aca="false">'1. Inputs'!H34</f>
         <v>0</v>
       </c>
       <c r="I7" s="11" t="n">
-        <f aca="false">'1. Inputs'!I33</f>
+        <f aca="false">'1. Inputs'!I34</f>
         <v>0</v>
       </c>
       <c r="J7" s="11" t="n">
-        <f aca="false">'1. Inputs'!J33</f>
+        <f aca="false">'1. Inputs'!J34</f>
         <v>0</v>
       </c>
       <c r="K7" s="11" t="n">
-        <f aca="false">'1. Inputs'!K33</f>
+        <f aca="false">'1. Inputs'!K34</f>
         <v>0</v>
       </c>
       <c r="L7" s="11" t="n">
-        <f aca="false">'1. Inputs'!L33</f>
+        <f aca="false">'1. Inputs'!L34</f>
         <v>0</v>
       </c>
     </row>
@@ -8222,43 +8457,43 @@
         <v>124</v>
       </c>
       <c r="C8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!B33=0,'1. Inputs'!B33=""),"-",('1. Inputs'!C33-'1. Inputs'!B33)/ABS('1. Inputs'!B33))</f>
+        <f aca="false">IF(OR('1. Inputs'!B34=0,'1. Inputs'!B34=""),"-",('1. Inputs'!C34-'1. Inputs'!B34)/ABS('1. Inputs'!B34))</f>
         <v>-</v>
       </c>
       <c r="D8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!C33=0,'1. Inputs'!C33=""),"-",('1. Inputs'!D33-'1. Inputs'!C33)/ABS('1. Inputs'!C33))</f>
+        <f aca="false">IF(OR('1. Inputs'!C34=0,'1. Inputs'!C34=""),"-",('1. Inputs'!D34-'1. Inputs'!C34)/ABS('1. Inputs'!C34))</f>
         <v>-</v>
       </c>
       <c r="E8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!D33=0,'1. Inputs'!D33=""),"-",('1. Inputs'!E33-'1. Inputs'!D33)/ABS('1. Inputs'!D33))</f>
+        <f aca="false">IF(OR('1. Inputs'!D34=0,'1. Inputs'!D34=""),"-",('1. Inputs'!E34-'1. Inputs'!D34)/ABS('1. Inputs'!D34))</f>
         <v>-</v>
       </c>
       <c r="F8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!E33=0,'1. Inputs'!E33=""),"-",('1. Inputs'!F33-'1. Inputs'!E33)/ABS('1. Inputs'!E33))</f>
+        <f aca="false">IF(OR('1. Inputs'!E34=0,'1. Inputs'!E34=""),"-",('1. Inputs'!F34-'1. Inputs'!E34)/ABS('1. Inputs'!E34))</f>
         <v>-</v>
       </c>
       <c r="G8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!F33=0,'1. Inputs'!F33=""),"-",('1. Inputs'!G33-'1. Inputs'!F33)/ABS('1. Inputs'!F33))</f>
+        <f aca="false">IF(OR('1. Inputs'!F34=0,'1. Inputs'!F34=""),"-",('1. Inputs'!G34-'1. Inputs'!F34)/ABS('1. Inputs'!F34))</f>
         <v>-</v>
       </c>
       <c r="H8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!G33=0,'1. Inputs'!G33=""),"-",('1. Inputs'!H33-'1. Inputs'!G33)/ABS('1. Inputs'!G33))</f>
+        <f aca="false">IF(OR('1. Inputs'!G34=0,'1. Inputs'!G34=""),"-",('1. Inputs'!H34-'1. Inputs'!G34)/ABS('1. Inputs'!G34))</f>
         <v>-</v>
       </c>
       <c r="I8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!H33=0,'1. Inputs'!H33=""),"-",('1. Inputs'!I33-'1. Inputs'!H33)/ABS('1. Inputs'!H33))</f>
+        <f aca="false">IF(OR('1. Inputs'!H34=0,'1. Inputs'!H34=""),"-",('1. Inputs'!I34-'1. Inputs'!H34)/ABS('1. Inputs'!H34))</f>
         <v>-</v>
       </c>
       <c r="J8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!I33=0,'1. Inputs'!I33=""),"-",('1. Inputs'!J33-'1. Inputs'!I33)/ABS('1. Inputs'!I33))</f>
+        <f aca="false">IF(OR('1. Inputs'!I34=0,'1. Inputs'!I34=""),"-",('1. Inputs'!J34-'1. Inputs'!I34)/ABS('1. Inputs'!I34))</f>
         <v>-</v>
       </c>
       <c r="K8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!J33=0,'1. Inputs'!J33=""),"-",('1. Inputs'!K33-'1. Inputs'!J33)/ABS('1. Inputs'!J33))</f>
+        <f aca="false">IF(OR('1. Inputs'!J34=0,'1. Inputs'!J34=""),"-",('1. Inputs'!K34-'1. Inputs'!J34)/ABS('1. Inputs'!J34))</f>
         <v>-</v>
       </c>
       <c r="L8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!K33=0,'1. Inputs'!K33=""),"-",('1. Inputs'!L33-'1. Inputs'!K33)/ABS('1. Inputs'!K33))</f>
+        <f aca="false">IF(OR('1. Inputs'!K34=0,'1. Inputs'!K34=""),"-",('1. Inputs'!L34-'1. Inputs'!K34)/ABS('1. Inputs'!K34))</f>
         <v>-</v>
       </c>
     </row>
@@ -8267,47 +8502,47 @@
         <v>139</v>
       </c>
       <c r="B9" s="11" t="n">
-        <f aca="false">'1. Inputs'!B34</f>
+        <f aca="false">'1. Inputs'!B35</f>
         <v>0</v>
       </c>
       <c r="C9" s="11" t="n">
-        <f aca="false">'1. Inputs'!C34</f>
+        <f aca="false">'1. Inputs'!C35</f>
         <v>0</v>
       </c>
       <c r="D9" s="11" t="n">
-        <f aca="false">'1. Inputs'!D34</f>
+        <f aca="false">'1. Inputs'!D35</f>
         <v>0</v>
       </c>
       <c r="E9" s="11" t="n">
-        <f aca="false">'1. Inputs'!E34</f>
+        <f aca="false">'1. Inputs'!E35</f>
         <v>0</v>
       </c>
       <c r="F9" s="11" t="n">
-        <f aca="false">'1. Inputs'!F34</f>
+        <f aca="false">'1. Inputs'!F35</f>
         <v>0</v>
       </c>
       <c r="G9" s="11" t="n">
-        <f aca="false">'1. Inputs'!G34</f>
+        <f aca="false">'1. Inputs'!G35</f>
         <v>0</v>
       </c>
       <c r="H9" s="11" t="n">
-        <f aca="false">'1. Inputs'!H34</f>
+        <f aca="false">'1. Inputs'!H35</f>
         <v>0</v>
       </c>
       <c r="I9" s="11" t="n">
-        <f aca="false">'1. Inputs'!I34</f>
+        <f aca="false">'1. Inputs'!I35</f>
         <v>0</v>
       </c>
       <c r="J9" s="11" t="n">
-        <f aca="false">'1. Inputs'!J34</f>
+        <f aca="false">'1. Inputs'!J35</f>
         <v>0</v>
       </c>
       <c r="K9" s="11" t="n">
-        <f aca="false">'1. Inputs'!K34</f>
+        <f aca="false">'1. Inputs'!K35</f>
         <v>0</v>
       </c>
       <c r="L9" s="11" t="n">
-        <f aca="false">'1. Inputs'!L34</f>
+        <f aca="false">'1. Inputs'!L35</f>
         <v>0</v>
       </c>
     </row>
@@ -8316,47 +8551,47 @@
         <v>140</v>
       </c>
       <c r="B10" s="11" t="n">
-        <f aca="false">'1. Inputs'!B35</f>
+        <f aca="false">'1. Inputs'!B36</f>
         <v>0</v>
       </c>
       <c r="C10" s="11" t="n">
-        <f aca="false">'1. Inputs'!C35</f>
+        <f aca="false">'1. Inputs'!C36</f>
         <v>0</v>
       </c>
       <c r="D10" s="11" t="n">
-        <f aca="false">'1. Inputs'!D35</f>
+        <f aca="false">'1. Inputs'!D36</f>
         <v>0</v>
       </c>
       <c r="E10" s="11" t="n">
-        <f aca="false">'1. Inputs'!E35</f>
+        <f aca="false">'1. Inputs'!E36</f>
         <v>0</v>
       </c>
       <c r="F10" s="11" t="n">
-        <f aca="false">'1. Inputs'!F35</f>
+        <f aca="false">'1. Inputs'!F36</f>
         <v>0</v>
       </c>
       <c r="G10" s="11" t="n">
-        <f aca="false">'1. Inputs'!G35</f>
+        <f aca="false">'1. Inputs'!G36</f>
         <v>0</v>
       </c>
       <c r="H10" s="11" t="n">
-        <f aca="false">'1. Inputs'!H35</f>
+        <f aca="false">'1. Inputs'!H36</f>
         <v>0</v>
       </c>
       <c r="I10" s="11" t="n">
-        <f aca="false">'1. Inputs'!I35</f>
+        <f aca="false">'1. Inputs'!I36</f>
         <v>0</v>
       </c>
       <c r="J10" s="11" t="n">
-        <f aca="false">'1. Inputs'!J35</f>
+        <f aca="false">'1. Inputs'!J36</f>
         <v>0</v>
       </c>
       <c r="K10" s="11" t="n">
-        <f aca="false">'1. Inputs'!K35</f>
+        <f aca="false">'1. Inputs'!K36</f>
         <v>0</v>
       </c>
       <c r="L10" s="11" t="n">
-        <f aca="false">'1. Inputs'!L35</f>
+        <f aca="false">'1. Inputs'!L36</f>
         <v>0</v>
       </c>
     </row>
@@ -8365,47 +8600,47 @@
         <v>141</v>
       </c>
       <c r="B11" s="11" t="n">
-        <f aca="false">'1. Inputs'!B34-'1. Inputs'!B35</f>
+        <f aca="false">'1. Inputs'!B35-'1. Inputs'!B36</f>
         <v>0</v>
       </c>
       <c r="C11" s="11" t="n">
-        <f aca="false">'1. Inputs'!C34-'1. Inputs'!C35</f>
+        <f aca="false">'1. Inputs'!C35-'1. Inputs'!C36</f>
         <v>0</v>
       </c>
       <c r="D11" s="11" t="n">
-        <f aca="false">'1. Inputs'!D34-'1. Inputs'!D35</f>
+        <f aca="false">'1. Inputs'!D35-'1. Inputs'!D36</f>
         <v>0</v>
       </c>
       <c r="E11" s="11" t="n">
-        <f aca="false">'1. Inputs'!E34-'1. Inputs'!E35</f>
+        <f aca="false">'1. Inputs'!E35-'1. Inputs'!E36</f>
         <v>0</v>
       </c>
       <c r="F11" s="11" t="n">
-        <f aca="false">'1. Inputs'!F34-'1. Inputs'!F35</f>
+        <f aca="false">'1. Inputs'!F35-'1. Inputs'!F36</f>
         <v>0</v>
       </c>
       <c r="G11" s="11" t="n">
-        <f aca="false">'1. Inputs'!G34-'1. Inputs'!G35</f>
+        <f aca="false">'1. Inputs'!G35-'1. Inputs'!G36</f>
         <v>0</v>
       </c>
       <c r="H11" s="11" t="n">
-        <f aca="false">'1. Inputs'!H34-'1. Inputs'!H35</f>
+        <f aca="false">'1. Inputs'!H35-'1. Inputs'!H36</f>
         <v>0</v>
       </c>
       <c r="I11" s="11" t="n">
-        <f aca="false">'1. Inputs'!I34-'1. Inputs'!I35</f>
+        <f aca="false">'1. Inputs'!I35-'1. Inputs'!I36</f>
         <v>0</v>
       </c>
       <c r="J11" s="11" t="n">
-        <f aca="false">'1. Inputs'!J34-'1. Inputs'!J35</f>
+        <f aca="false">'1. Inputs'!J35-'1. Inputs'!J36</f>
         <v>0</v>
       </c>
       <c r="K11" s="11" t="n">
-        <f aca="false">'1. Inputs'!K34-'1. Inputs'!K35</f>
+        <f aca="false">'1. Inputs'!K35-'1. Inputs'!K36</f>
         <v>0</v>
       </c>
       <c r="L11" s="11" t="n">
-        <f aca="false">'1. Inputs'!L34-'1. Inputs'!L35</f>
+        <f aca="false">'1. Inputs'!L35-'1. Inputs'!L36</f>
         <v>0</v>
       </c>
     </row>
@@ -8414,47 +8649,47 @@
         <v>142</v>
       </c>
       <c r="B12" s="11" t="n">
-        <f aca="false">'1. Inputs'!B36</f>
+        <f aca="false">'1. Inputs'!B37</f>
         <v>0</v>
       </c>
       <c r="C12" s="11" t="n">
-        <f aca="false">'1. Inputs'!C36</f>
+        <f aca="false">'1. Inputs'!C37</f>
         <v>0</v>
       </c>
       <c r="D12" s="11" t="n">
-        <f aca="false">'1. Inputs'!D36</f>
+        <f aca="false">'1. Inputs'!D37</f>
         <v>0</v>
       </c>
       <c r="E12" s="11" t="n">
-        <f aca="false">'1. Inputs'!E36</f>
+        <f aca="false">'1. Inputs'!E37</f>
         <v>0</v>
       </c>
       <c r="F12" s="11" t="n">
-        <f aca="false">'1. Inputs'!F36</f>
+        <f aca="false">'1. Inputs'!F37</f>
         <v>0</v>
       </c>
       <c r="G12" s="11" t="n">
-        <f aca="false">'1. Inputs'!G36</f>
+        <f aca="false">'1. Inputs'!G37</f>
         <v>0</v>
       </c>
       <c r="H12" s="11" t="n">
-        <f aca="false">'1. Inputs'!H36</f>
+        <f aca="false">'1. Inputs'!H37</f>
         <v>0</v>
       </c>
       <c r="I12" s="11" t="n">
-        <f aca="false">'1. Inputs'!I36</f>
+        <f aca="false">'1. Inputs'!I37</f>
         <v>0</v>
       </c>
       <c r="J12" s="11" t="n">
-        <f aca="false">'1. Inputs'!J36</f>
+        <f aca="false">'1. Inputs'!J37</f>
         <v>0</v>
       </c>
       <c r="K12" s="11" t="n">
-        <f aca="false">'1. Inputs'!K36</f>
+        <f aca="false">'1. Inputs'!K37</f>
         <v>0</v>
       </c>
       <c r="L12" s="11" t="n">
-        <f aca="false">'1. Inputs'!L36</f>
+        <f aca="false">'1. Inputs'!L37</f>
         <v>0</v>
       </c>
     </row>
@@ -8463,47 +8698,47 @@
         <v>82</v>
       </c>
       <c r="B13" s="11" t="n">
-        <f aca="false">'1. Inputs'!B38</f>
+        <f aca="false">'1. Inputs'!B39</f>
         <v>0</v>
       </c>
       <c r="C13" s="11" t="n">
-        <f aca="false">'1. Inputs'!C38</f>
+        <f aca="false">'1. Inputs'!C39</f>
         <v>0</v>
       </c>
       <c r="D13" s="11" t="n">
-        <f aca="false">'1. Inputs'!D38</f>
+        <f aca="false">'1. Inputs'!D39</f>
         <v>0</v>
       </c>
       <c r="E13" s="11" t="n">
-        <f aca="false">'1. Inputs'!E38</f>
+        <f aca="false">'1. Inputs'!E39</f>
         <v>0</v>
       </c>
       <c r="F13" s="11" t="n">
-        <f aca="false">'1. Inputs'!F38</f>
+        <f aca="false">'1. Inputs'!F39</f>
         <v>0</v>
       </c>
       <c r="G13" s="11" t="n">
-        <f aca="false">'1. Inputs'!G38</f>
+        <f aca="false">'1. Inputs'!G39</f>
         <v>0</v>
       </c>
       <c r="H13" s="11" t="n">
-        <f aca="false">'1. Inputs'!H38</f>
+        <f aca="false">'1. Inputs'!H39</f>
         <v>0</v>
       </c>
       <c r="I13" s="11" t="n">
-        <f aca="false">'1. Inputs'!I38</f>
+        <f aca="false">'1. Inputs'!I39</f>
         <v>0</v>
       </c>
       <c r="J13" s="11" t="n">
-        <f aca="false">'1. Inputs'!J38</f>
+        <f aca="false">'1. Inputs'!J39</f>
         <v>0</v>
       </c>
       <c r="K13" s="11" t="n">
-        <f aca="false">'1. Inputs'!K38</f>
+        <f aca="false">'1. Inputs'!K39</f>
         <v>0</v>
       </c>
       <c r="L13" s="11" t="n">
-        <f aca="false">'1. Inputs'!L38</f>
+        <f aca="false">'1. Inputs'!L39</f>
         <v>0</v>
       </c>
     </row>
@@ -8515,43 +8750,43 @@
         <v>124</v>
       </c>
       <c r="C14" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!B38=0,'1. Inputs'!B38=""),"-",('1. Inputs'!C38-'1. Inputs'!B38)/ABS('1. Inputs'!B38))</f>
+        <f aca="false">IF(OR('1. Inputs'!B39=0,'1. Inputs'!B39=""),"-",('1. Inputs'!C39-'1. Inputs'!B39)/ABS('1. Inputs'!B39))</f>
         <v>-</v>
       </c>
       <c r="D14" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!C38=0,'1. Inputs'!C38=""),"-",('1. Inputs'!D38-'1. Inputs'!C38)/ABS('1. Inputs'!C38))</f>
+        <f aca="false">IF(OR('1. Inputs'!C39=0,'1. Inputs'!C39=""),"-",('1. Inputs'!D39-'1. Inputs'!C39)/ABS('1. Inputs'!C39))</f>
         <v>-</v>
       </c>
       <c r="E14" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!D38=0,'1. Inputs'!D38=""),"-",('1. Inputs'!E38-'1. Inputs'!D38)/ABS('1. Inputs'!D38))</f>
+        <f aca="false">IF(OR('1. Inputs'!D39=0,'1. Inputs'!D39=""),"-",('1. Inputs'!E39-'1. Inputs'!D39)/ABS('1. Inputs'!D39))</f>
         <v>-</v>
       </c>
       <c r="F14" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!E38=0,'1. Inputs'!E38=""),"-",('1. Inputs'!F38-'1. Inputs'!E38)/ABS('1. Inputs'!E38))</f>
+        <f aca="false">IF(OR('1. Inputs'!E39=0,'1. Inputs'!E39=""),"-",('1. Inputs'!F39-'1. Inputs'!E39)/ABS('1. Inputs'!E39))</f>
         <v>-</v>
       </c>
       <c r="G14" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!F38=0,'1. Inputs'!F38=""),"-",('1. Inputs'!G38-'1. Inputs'!F38)/ABS('1. Inputs'!F38))</f>
+        <f aca="false">IF(OR('1. Inputs'!F39=0,'1. Inputs'!F39=""),"-",('1. Inputs'!G39-'1. Inputs'!F39)/ABS('1. Inputs'!F39))</f>
         <v>-</v>
       </c>
       <c r="H14" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!G38=0,'1. Inputs'!G38=""),"-",('1. Inputs'!H38-'1. Inputs'!G38)/ABS('1. Inputs'!G38))</f>
+        <f aca="false">IF(OR('1. Inputs'!G39=0,'1. Inputs'!G39=""),"-",('1. Inputs'!H39-'1. Inputs'!G39)/ABS('1. Inputs'!G39))</f>
         <v>-</v>
       </c>
       <c r="I14" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!H38=0,'1. Inputs'!H38=""),"-",('1. Inputs'!I38-'1. Inputs'!H38)/ABS('1. Inputs'!H38))</f>
+        <f aca="false">IF(OR('1. Inputs'!H39=0,'1. Inputs'!H39=""),"-",('1. Inputs'!I39-'1. Inputs'!H39)/ABS('1. Inputs'!H39))</f>
         <v>-</v>
       </c>
       <c r="J14" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!I38=0,'1. Inputs'!I38=""),"-",('1. Inputs'!J38-'1. Inputs'!I38)/ABS('1. Inputs'!I38))</f>
+        <f aca="false">IF(OR('1. Inputs'!I39=0,'1. Inputs'!I39=""),"-",('1. Inputs'!J39-'1. Inputs'!I39)/ABS('1. Inputs'!I39))</f>
         <v>-</v>
       </c>
       <c r="K14" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!J38=0,'1. Inputs'!J38=""),"-",('1. Inputs'!K38-'1. Inputs'!J38)/ABS('1. Inputs'!J38))</f>
+        <f aca="false">IF(OR('1. Inputs'!J39=0,'1. Inputs'!J39=""),"-",('1. Inputs'!K39-'1. Inputs'!J39)/ABS('1. Inputs'!J39))</f>
         <v>-</v>
       </c>
       <c r="L14" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!K38=0,'1. Inputs'!K38=""),"-",('1. Inputs'!L38-'1. Inputs'!K38)/ABS('1. Inputs'!K38))</f>
+        <f aca="false">IF(OR('1. Inputs'!K39=0,'1. Inputs'!K39=""),"-",('1. Inputs'!L39-'1. Inputs'!K39)/ABS('1. Inputs'!K39))</f>
         <v>-</v>
       </c>
     </row>
@@ -8560,47 +8795,47 @@
         <v>144</v>
       </c>
       <c r="B15" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!B33-'1. Inputs'!B36)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!B34-'1. Inputs'!B37)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="C15" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!C33-'1. Inputs'!C36)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!C34-'1. Inputs'!C37)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="D15" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!D33-'1. Inputs'!D36)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!D34-'1. Inputs'!D37)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="E15" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!E33-'1. Inputs'!E36)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!E34-'1. Inputs'!E37)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="F15" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!F33-'1. Inputs'!F36)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!F34-'1. Inputs'!F37)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="G15" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!G33-'1. Inputs'!G36)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!G34-'1. Inputs'!G37)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="H15" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!H33-'1. Inputs'!H36)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!H34-'1. Inputs'!H37)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="I15" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!I33-'1. Inputs'!I36)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!I34-'1. Inputs'!I37)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="J15" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!J33-'1. Inputs'!J36)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!J34-'1. Inputs'!J37)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="K15" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!K33-'1. Inputs'!K36)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!K34-'1. Inputs'!K37)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="L15" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!L33-'1. Inputs'!L36)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!L34-'1. Inputs'!L37)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
     </row>
@@ -8609,47 +8844,47 @@
         <v>145</v>
       </c>
       <c r="B16" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!B33=0,'1. Inputs'!B33=""),"-",'1. Inputs'!B34/'1. Inputs'!B33)</f>
+        <f aca="false">IF(OR('1. Inputs'!B34=0,'1. Inputs'!B34=""),"-",'1. Inputs'!B35/'1. Inputs'!B34)</f>
         <v>-</v>
       </c>
       <c r="C16" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!C33=0,'1. Inputs'!C33=""),"-",'1. Inputs'!C34/'1. Inputs'!C33)</f>
+        <f aca="false">IF(OR('1. Inputs'!C34=0,'1. Inputs'!C34=""),"-",'1. Inputs'!C35/'1. Inputs'!C34)</f>
         <v>-</v>
       </c>
       <c r="D16" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!D33=0,'1. Inputs'!D33=""),"-",'1. Inputs'!D34/'1. Inputs'!D33)</f>
+        <f aca="false">IF(OR('1. Inputs'!D34=0,'1. Inputs'!D34=""),"-",'1. Inputs'!D35/'1. Inputs'!D34)</f>
         <v>-</v>
       </c>
       <c r="E16" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!E33=0,'1. Inputs'!E33=""),"-",'1. Inputs'!E34/'1. Inputs'!E33)</f>
+        <f aca="false">IF(OR('1. Inputs'!E34=0,'1. Inputs'!E34=""),"-",'1. Inputs'!E35/'1. Inputs'!E34)</f>
         <v>-</v>
       </c>
       <c r="F16" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!F33=0,'1. Inputs'!F33=""),"-",'1. Inputs'!F34/'1. Inputs'!F33)</f>
+        <f aca="false">IF(OR('1. Inputs'!F34=0,'1. Inputs'!F34=""),"-",'1. Inputs'!F35/'1. Inputs'!F34)</f>
         <v>-</v>
       </c>
       <c r="G16" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!G33=0,'1. Inputs'!G33=""),"-",'1. Inputs'!G34/'1. Inputs'!G33)</f>
+        <f aca="false">IF(OR('1. Inputs'!G34=0,'1. Inputs'!G34=""),"-",'1. Inputs'!G35/'1. Inputs'!G34)</f>
         <v>-</v>
       </c>
       <c r="H16" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!H33=0,'1. Inputs'!H33=""),"-",'1. Inputs'!H34/'1. Inputs'!H33)</f>
+        <f aca="false">IF(OR('1. Inputs'!H34=0,'1. Inputs'!H34=""),"-",'1. Inputs'!H35/'1. Inputs'!H34)</f>
         <v>-</v>
       </c>
       <c r="I16" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!I33=0,'1. Inputs'!I33=""),"-",'1. Inputs'!I34/'1. Inputs'!I33)</f>
+        <f aca="false">IF(OR('1. Inputs'!I34=0,'1. Inputs'!I34=""),"-",'1. Inputs'!I35/'1. Inputs'!I34)</f>
         <v>-</v>
       </c>
       <c r="J16" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!J33=0,'1. Inputs'!J33=""),"-",'1. Inputs'!J34/'1. Inputs'!J33)</f>
+        <f aca="false">IF(OR('1. Inputs'!J34=0,'1. Inputs'!J34=""),"-",'1. Inputs'!J35/'1. Inputs'!J34)</f>
         <v>-</v>
       </c>
       <c r="K16" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!K33=0,'1. Inputs'!K33=""),"-",'1. Inputs'!K34/'1. Inputs'!K33)</f>
+        <f aca="false">IF(OR('1. Inputs'!K34=0,'1. Inputs'!K34=""),"-",'1. Inputs'!K35/'1. Inputs'!K34)</f>
         <v>-</v>
       </c>
       <c r="L16" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!L33=0,'1. Inputs'!L33=""),"-",'1. Inputs'!L34/'1. Inputs'!L33)</f>
+        <f aca="false">IF(OR('1. Inputs'!L34=0,'1. Inputs'!L34=""),"-",'1. Inputs'!L35/'1. Inputs'!L34)</f>
         <v>-</v>
       </c>
     </row>
@@ -8658,47 +8893,47 @@
         <v>146</v>
       </c>
       <c r="B17" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!B13=0,'1. Inputs'!B13=""),"-",'1. Inputs'!B34/'1. Inputs'!B13)</f>
+        <f aca="false">IF(OR('1. Inputs'!B13=0,'1. Inputs'!B13=""),"-",'1. Inputs'!B35/'1. Inputs'!B13)</f>
         <v>-</v>
       </c>
       <c r="C17" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!C13=0,'1. Inputs'!C13=""),"-",'1. Inputs'!C34/'1. Inputs'!C13)</f>
+        <f aca="false">IF(OR('1. Inputs'!C13=0,'1. Inputs'!C13=""),"-",'1. Inputs'!C35/'1. Inputs'!C13)</f>
         <v>-</v>
       </c>
       <c r="D17" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!D13=0,'1. Inputs'!D13=""),"-",'1. Inputs'!D34/'1. Inputs'!D13)</f>
+        <f aca="false">IF(OR('1. Inputs'!D13=0,'1. Inputs'!D13=""),"-",'1. Inputs'!D35/'1. Inputs'!D13)</f>
         <v>-</v>
       </c>
       <c r="E17" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!E13=0,'1. Inputs'!E13=""),"-",'1. Inputs'!E34/'1. Inputs'!E13)</f>
+        <f aca="false">IF(OR('1. Inputs'!E13=0,'1. Inputs'!E13=""),"-",'1. Inputs'!E35/'1. Inputs'!E13)</f>
         <v>-</v>
       </c>
       <c r="F17" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!F13=0,'1. Inputs'!F13=""),"-",'1. Inputs'!F34/'1. Inputs'!F13)</f>
+        <f aca="false">IF(OR('1. Inputs'!F13=0,'1. Inputs'!F13=""),"-",'1. Inputs'!F35/'1. Inputs'!F13)</f>
         <v>-</v>
       </c>
       <c r="G17" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!G13=0,'1. Inputs'!G13=""),"-",'1. Inputs'!G34/'1. Inputs'!G13)</f>
+        <f aca="false">IF(OR('1. Inputs'!G13=0,'1. Inputs'!G13=""),"-",'1. Inputs'!G35/'1. Inputs'!G13)</f>
         <v>-</v>
       </c>
       <c r="H17" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!H13=0,'1. Inputs'!H13=""),"-",'1. Inputs'!H34/'1. Inputs'!H13)</f>
+        <f aca="false">IF(OR('1. Inputs'!H13=0,'1. Inputs'!H13=""),"-",'1. Inputs'!H35/'1. Inputs'!H13)</f>
         <v>-</v>
       </c>
       <c r="I17" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!I13=0,'1. Inputs'!I13=""),"-",'1. Inputs'!I34/'1. Inputs'!I13)</f>
+        <f aca="false">IF(OR('1. Inputs'!I13=0,'1. Inputs'!I13=""),"-",'1. Inputs'!I35/'1. Inputs'!I13)</f>
         <v>-</v>
       </c>
       <c r="J17" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!J13=0,'1. Inputs'!J13=""),"-",'1. Inputs'!J34/'1. Inputs'!J13)</f>
+        <f aca="false">IF(OR('1. Inputs'!J13=0,'1. Inputs'!J13=""),"-",'1. Inputs'!J35/'1. Inputs'!J13)</f>
         <v>-</v>
       </c>
       <c r="K17" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!K13=0,'1. Inputs'!K13=""),"-",'1. Inputs'!K34/'1. Inputs'!K13)</f>
+        <f aca="false">IF(OR('1. Inputs'!K13=0,'1. Inputs'!K13=""),"-",'1. Inputs'!K35/'1. Inputs'!K13)</f>
         <v>-</v>
       </c>
       <c r="L17" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!L13=0,'1. Inputs'!L13=""),"-",'1. Inputs'!L34/'1. Inputs'!L13)</f>
+        <f aca="false">IF(OR('1. Inputs'!L13=0,'1. Inputs'!L13=""),"-",'1. Inputs'!L35/'1. Inputs'!L13)</f>
         <v>-</v>
       </c>
     </row>
@@ -8707,47 +8942,47 @@
         <v>147</v>
       </c>
       <c r="B18" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!B13=0,'1. Inputs'!B13=""),"-",('1. Inputs'!B34-'1. Inputs'!B35)/'1. Inputs'!B13)</f>
+        <f aca="false">IF(OR('1. Inputs'!B13=0,'1. Inputs'!B13=""),"-",('1. Inputs'!B35-'1. Inputs'!B36)/'1. Inputs'!B13)</f>
         <v>-</v>
       </c>
       <c r="C18" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!C13=0,'1. Inputs'!C13=""),"-",('1. Inputs'!C34-'1. Inputs'!C35)/'1. Inputs'!C13)</f>
+        <f aca="false">IF(OR('1. Inputs'!C13=0,'1. Inputs'!C13=""),"-",('1. Inputs'!C35-'1. Inputs'!C36)/'1. Inputs'!C13)</f>
         <v>-</v>
       </c>
       <c r="D18" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!D13=0,'1. Inputs'!D13=""),"-",('1. Inputs'!D34-'1. Inputs'!D35)/'1. Inputs'!D13)</f>
+        <f aca="false">IF(OR('1. Inputs'!D13=0,'1. Inputs'!D13=""),"-",('1. Inputs'!D35-'1. Inputs'!D36)/'1. Inputs'!D13)</f>
         <v>-</v>
       </c>
       <c r="E18" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!E13=0,'1. Inputs'!E13=""),"-",('1. Inputs'!E34-'1. Inputs'!E35)/'1. Inputs'!E13)</f>
+        <f aca="false">IF(OR('1. Inputs'!E13=0,'1. Inputs'!E13=""),"-",('1. Inputs'!E35-'1. Inputs'!E36)/'1. Inputs'!E13)</f>
         <v>-</v>
       </c>
       <c r="F18" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!F13=0,'1. Inputs'!F13=""),"-",('1. Inputs'!F34-'1. Inputs'!F35)/'1. Inputs'!F13)</f>
+        <f aca="false">IF(OR('1. Inputs'!F13=0,'1. Inputs'!F13=""),"-",('1. Inputs'!F35-'1. Inputs'!F36)/'1. Inputs'!F13)</f>
         <v>-</v>
       </c>
       <c r="G18" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!G13=0,'1. Inputs'!G13=""),"-",('1. Inputs'!G34-'1. Inputs'!G35)/'1. Inputs'!G13)</f>
+        <f aca="false">IF(OR('1. Inputs'!G13=0,'1. Inputs'!G13=""),"-",('1. Inputs'!G35-'1. Inputs'!G36)/'1. Inputs'!G13)</f>
         <v>-</v>
       </c>
       <c r="H18" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!H13=0,'1. Inputs'!H13=""),"-",('1. Inputs'!H34-'1. Inputs'!H35)/'1. Inputs'!H13)</f>
+        <f aca="false">IF(OR('1. Inputs'!H13=0,'1. Inputs'!H13=""),"-",('1. Inputs'!H35-'1. Inputs'!H36)/'1. Inputs'!H13)</f>
         <v>-</v>
       </c>
       <c r="I18" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!I13=0,'1. Inputs'!I13=""),"-",('1. Inputs'!I34-'1. Inputs'!I35)/'1. Inputs'!I13)</f>
+        <f aca="false">IF(OR('1. Inputs'!I13=0,'1. Inputs'!I13=""),"-",('1. Inputs'!I35-'1. Inputs'!I36)/'1. Inputs'!I13)</f>
         <v>-</v>
       </c>
       <c r="J18" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!J13=0,'1. Inputs'!J13=""),"-",('1. Inputs'!J34-'1. Inputs'!J35)/'1. Inputs'!J13)</f>
+        <f aca="false">IF(OR('1. Inputs'!J13=0,'1. Inputs'!J13=""),"-",('1. Inputs'!J35-'1. Inputs'!J36)/'1. Inputs'!J13)</f>
         <v>-</v>
       </c>
       <c r="K18" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!K13=0,'1. Inputs'!K13=""),"-",('1. Inputs'!K34-'1. Inputs'!K35)/'1. Inputs'!K13)</f>
+        <f aca="false">IF(OR('1. Inputs'!K13=0,'1. Inputs'!K13=""),"-",('1. Inputs'!K35-'1. Inputs'!K36)/'1. Inputs'!K13)</f>
         <v>-</v>
       </c>
       <c r="L18" s="13" t="str">
-        <f aca="false">IF(OR('1. Inputs'!L13=0,'1. Inputs'!L13=""),"-",('1. Inputs'!L34-'1. Inputs'!L35)/'1. Inputs'!L13)</f>
+        <f aca="false">IF(OR('1. Inputs'!L13=0,'1. Inputs'!L13=""),"-",('1. Inputs'!L35-'1. Inputs'!L36)/'1. Inputs'!L13)</f>
         <v>-</v>
       </c>
     </row>
@@ -8846,49 +9081,49 @@
       <c r="A4" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="B4" s="11" t="str">
-        <f aca="false">'1. Inputs'!B53</f>
-        <v>FY1 (Oldest)</v>
-      </c>
-      <c r="C4" s="11" t="str">
-        <f aca="false">'1. Inputs'!C53</f>
-        <v>FY2</v>
-      </c>
-      <c r="D4" s="11" t="str">
-        <f aca="false">'1. Inputs'!D53</f>
-        <v>FY3</v>
-      </c>
-      <c r="E4" s="11" t="str">
-        <f aca="false">'1. Inputs'!E53</f>
-        <v>FY4</v>
-      </c>
-      <c r="F4" s="11" t="str">
-        <f aca="false">'1. Inputs'!F53</f>
-        <v>FY5</v>
-      </c>
-      <c r="G4" s="11" t="str">
-        <f aca="false">'1. Inputs'!G53</f>
-        <v>FY6</v>
-      </c>
-      <c r="H4" s="11" t="str">
-        <f aca="false">'1. Inputs'!H53</f>
-        <v>FY7</v>
-      </c>
-      <c r="I4" s="11" t="str">
-        <f aca="false">'1. Inputs'!I53</f>
-        <v>FY8</v>
-      </c>
-      <c r="J4" s="11" t="str">
-        <f aca="false">'1. Inputs'!J53</f>
-        <v>FY9</v>
-      </c>
-      <c r="K4" s="11" t="str">
-        <f aca="false">'1. Inputs'!K53</f>
-        <v>FY10 (Latest)</v>
-      </c>
-      <c r="L4" s="11" t="str">
-        <f aca="false">'1. Inputs'!L53</f>
-        <v>TTM</v>
+      <c r="B4" s="11" t="n">
+        <f aca="false">'1. Inputs'!B54</f>
+        <v>0</v>
+      </c>
+      <c r="C4" s="11" t="n">
+        <f aca="false">'1. Inputs'!C54</f>
+        <v>0</v>
+      </c>
+      <c r="D4" s="11" t="n">
+        <f aca="false">'1. Inputs'!D54</f>
+        <v>0</v>
+      </c>
+      <c r="E4" s="11" t="n">
+        <f aca="false">'1. Inputs'!E54</f>
+        <v>0</v>
+      </c>
+      <c r="F4" s="11" t="n">
+        <f aca="false">'1. Inputs'!F54</f>
+        <v>0</v>
+      </c>
+      <c r="G4" s="11" t="n">
+        <f aca="false">'1. Inputs'!G54</f>
+        <v>0</v>
+      </c>
+      <c r="H4" s="11" t="n">
+        <f aca="false">'1. Inputs'!H54</f>
+        <v>0</v>
+      </c>
+      <c r="I4" s="11" t="n">
+        <f aca="false">'1. Inputs'!I54</f>
+        <v>0</v>
+      </c>
+      <c r="J4" s="11" t="n">
+        <f aca="false">'1. Inputs'!J54</f>
+        <v>0</v>
+      </c>
+      <c r="K4" s="11" t="n">
+        <f aca="false">'1. Inputs'!K54</f>
+        <v>0</v>
+      </c>
+      <c r="L4" s="11" t="n">
+        <f aca="false">'1. Inputs'!L54</f>
+        <v>0</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8898,45 +9133,45 @@
       <c r="B5" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="C5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!B53=0,'1. Inputs'!B53=""),"-",('1. Inputs'!C53-'1. Inputs'!B53)/ABS('1. Inputs'!B53))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!C53=0,'1. Inputs'!C53=""),"-",('1. Inputs'!D53-'1. Inputs'!C53)/ABS('1. Inputs'!C53))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!D53=0,'1. Inputs'!D53=""),"-",('1. Inputs'!E53-'1. Inputs'!D53)/ABS('1. Inputs'!D53))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!E53=0,'1. Inputs'!E53=""),"-",('1. Inputs'!F53-'1. Inputs'!E53)/ABS('1. Inputs'!E53))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!F53=0,'1. Inputs'!F53=""),"-",('1. Inputs'!G53-'1. Inputs'!F53)/ABS('1. Inputs'!F53))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="H5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!G53=0,'1. Inputs'!G53=""),"-",('1. Inputs'!H53-'1. Inputs'!G53)/ABS('1. Inputs'!G53))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!H53=0,'1. Inputs'!H53=""),"-",('1. Inputs'!I53-'1. Inputs'!H53)/ABS('1. Inputs'!H53))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="J5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!I53=0,'1. Inputs'!I53=""),"-",('1. Inputs'!J53-'1. Inputs'!I53)/ABS('1. Inputs'!I53))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!J53=0,'1. Inputs'!J53=""),"-",('1. Inputs'!K53-'1. Inputs'!J53)/ABS('1. Inputs'!J53))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!K53=0,'1. Inputs'!K53=""),"-",('1. Inputs'!L53-'1. Inputs'!K53)/ABS('1. Inputs'!K53))</f>
-        <v>#VALUE!</v>
+      <c r="C5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!B54=0,'1. Inputs'!B54=""),"-",('1. Inputs'!C54-'1. Inputs'!B54)/ABS('1. Inputs'!B54))</f>
+        <v>-</v>
+      </c>
+      <c r="D5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!C54=0,'1. Inputs'!C54=""),"-",('1. Inputs'!D54-'1. Inputs'!C54)/ABS('1. Inputs'!C54))</f>
+        <v>-</v>
+      </c>
+      <c r="E5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!D54=0,'1. Inputs'!D54=""),"-",('1. Inputs'!E54-'1. Inputs'!D54)/ABS('1. Inputs'!D54))</f>
+        <v>-</v>
+      </c>
+      <c r="F5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!E54=0,'1. Inputs'!E54=""),"-",('1. Inputs'!F54-'1. Inputs'!E54)/ABS('1. Inputs'!E54))</f>
+        <v>-</v>
+      </c>
+      <c r="G5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!F54=0,'1. Inputs'!F54=""),"-",('1. Inputs'!G54-'1. Inputs'!F54)/ABS('1. Inputs'!F54))</f>
+        <v>-</v>
+      </c>
+      <c r="H5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!G54=0,'1. Inputs'!G54=""),"-",('1. Inputs'!H54-'1. Inputs'!G54)/ABS('1. Inputs'!G54))</f>
+        <v>-</v>
+      </c>
+      <c r="I5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!H54=0,'1. Inputs'!H54=""),"-",('1. Inputs'!I54-'1. Inputs'!H54)/ABS('1. Inputs'!H54))</f>
+        <v>-</v>
+      </c>
+      <c r="J5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!I54=0,'1. Inputs'!I54=""),"-",('1. Inputs'!J54-'1. Inputs'!I54)/ABS('1. Inputs'!I54))</f>
+        <v>-</v>
+      </c>
+      <c r="K5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!J54=0,'1. Inputs'!J54=""),"-",('1. Inputs'!K54-'1. Inputs'!J54)/ABS('1. Inputs'!J54))</f>
+        <v>-</v>
+      </c>
+      <c r="L5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!K54=0,'1. Inputs'!K54=""),"-",('1. Inputs'!L54-'1. Inputs'!K54)/ABS('1. Inputs'!K54))</f>
+        <v>-</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8944,47 +9179,47 @@
         <v>151</v>
       </c>
       <c r="B6" s="11" t="n">
-        <f aca="false">'1. Inputs'!B54</f>
+        <f aca="false">'1. Inputs'!B55</f>
         <v>0</v>
       </c>
       <c r="C6" s="11" t="n">
-        <f aca="false">'1. Inputs'!C54</f>
+        <f aca="false">'1. Inputs'!C55</f>
         <v>0</v>
       </c>
       <c r="D6" s="11" t="n">
-        <f aca="false">'1. Inputs'!D54</f>
+        <f aca="false">'1. Inputs'!D55</f>
         <v>0</v>
       </c>
       <c r="E6" s="11" t="n">
-        <f aca="false">'1. Inputs'!E54</f>
+        <f aca="false">'1. Inputs'!E55</f>
         <v>0</v>
       </c>
       <c r="F6" s="11" t="n">
-        <f aca="false">'1. Inputs'!F54</f>
+        <f aca="false">'1. Inputs'!F55</f>
         <v>0</v>
       </c>
       <c r="G6" s="11" t="n">
-        <f aca="false">'1. Inputs'!G54</f>
+        <f aca="false">'1. Inputs'!G55</f>
         <v>0</v>
       </c>
       <c r="H6" s="11" t="n">
-        <f aca="false">'1. Inputs'!H54</f>
+        <f aca="false">'1. Inputs'!H55</f>
         <v>0</v>
       </c>
       <c r="I6" s="11" t="n">
-        <f aca="false">'1. Inputs'!I54</f>
+        <f aca="false">'1. Inputs'!I55</f>
         <v>0</v>
       </c>
       <c r="J6" s="11" t="n">
-        <f aca="false">'1. Inputs'!J54</f>
+        <f aca="false">'1. Inputs'!J55</f>
         <v>0</v>
       </c>
       <c r="K6" s="11" t="n">
-        <f aca="false">'1. Inputs'!K54</f>
+        <f aca="false">'1. Inputs'!K55</f>
         <v>0</v>
       </c>
       <c r="L6" s="11" t="n">
-        <f aca="false">'1. Inputs'!L54</f>
+        <f aca="false">'1. Inputs'!L55</f>
         <v>0</v>
       </c>
     </row>
@@ -8992,49 +9227,49 @@
       <c r="A7" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="B7" s="11" t="e">
-        <f aca="false">'1. Inputs'!B53+'1. Inputs'!B54</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C7" s="11" t="e">
-        <f aca="false">'1. Inputs'!C53+'1. Inputs'!C54</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D7" s="11" t="e">
-        <f aca="false">'1. Inputs'!D53+'1. Inputs'!D54</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E7" s="11" t="e">
-        <f aca="false">'1. Inputs'!E53+'1. Inputs'!E54</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F7" s="11" t="e">
-        <f aca="false">'1. Inputs'!F53+'1. Inputs'!F54</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G7" s="11" t="e">
-        <f aca="false">'1. Inputs'!G53+'1. Inputs'!G54</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="H7" s="11" t="e">
-        <f aca="false">'1. Inputs'!H53+'1. Inputs'!H54</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I7" s="11" t="e">
-        <f aca="false">'1. Inputs'!I53+'1. Inputs'!I54</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="J7" s="11" t="e">
-        <f aca="false">'1. Inputs'!J53+'1. Inputs'!J54</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K7" s="11" t="e">
-        <f aca="false">'1. Inputs'!K53+'1. Inputs'!K54</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L7" s="11" t="e">
-        <f aca="false">'1. Inputs'!L53+'1. Inputs'!L54</f>
-        <v>#VALUE!</v>
+      <c r="B7" s="11" t="n">
+        <f aca="false">'1. Inputs'!B54+'1. Inputs'!B55</f>
+        <v>0</v>
+      </c>
+      <c r="C7" s="11" t="n">
+        <f aca="false">'1. Inputs'!C54+'1. Inputs'!C55</f>
+        <v>0</v>
+      </c>
+      <c r="D7" s="11" t="n">
+        <f aca="false">'1. Inputs'!D54+'1. Inputs'!D55</f>
+        <v>0</v>
+      </c>
+      <c r="E7" s="11" t="n">
+        <f aca="false">'1. Inputs'!E54+'1. Inputs'!E55</f>
+        <v>0</v>
+      </c>
+      <c r="F7" s="11" t="n">
+        <f aca="false">'1. Inputs'!F54+'1. Inputs'!F55</f>
+        <v>0</v>
+      </c>
+      <c r="G7" s="11" t="n">
+        <f aca="false">'1. Inputs'!G54+'1. Inputs'!G55</f>
+        <v>0</v>
+      </c>
+      <c r="H7" s="11" t="n">
+        <f aca="false">'1. Inputs'!H54+'1. Inputs'!H55</f>
+        <v>0</v>
+      </c>
+      <c r="I7" s="11" t="n">
+        <f aca="false">'1. Inputs'!I54+'1. Inputs'!I55</f>
+        <v>0</v>
+      </c>
+      <c r="J7" s="11" t="n">
+        <f aca="false">'1. Inputs'!J54+'1. Inputs'!J55</f>
+        <v>0</v>
+      </c>
+      <c r="K7" s="11" t="n">
+        <f aca="false">'1. Inputs'!K54+'1. Inputs'!K55</f>
+        <v>0</v>
+      </c>
+      <c r="L7" s="11" t="n">
+        <f aca="false">'1. Inputs'!L54+'1. Inputs'!L55</f>
+        <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9042,47 +9277,47 @@
         <v>153</v>
       </c>
       <c r="B8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!B12=0,'1. Inputs'!B12=""),"-",('1. Inputs'!B53+'1. Inputs'!B54)/'1. Inputs'!B12)</f>
+        <f aca="false">IF(OR('1. Inputs'!B12=0,'1. Inputs'!B12=""),"-",('1. Inputs'!B54+'1. Inputs'!B55)/'1. Inputs'!B12)</f>
         <v>-</v>
       </c>
       <c r="C8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!C12=0,'1. Inputs'!C12=""),"-",('1. Inputs'!C53+'1. Inputs'!C54)/'1. Inputs'!C12)</f>
+        <f aca="false">IF(OR('1. Inputs'!C12=0,'1. Inputs'!C12=""),"-",('1. Inputs'!C54+'1. Inputs'!C55)/'1. Inputs'!C12)</f>
         <v>-</v>
       </c>
       <c r="D8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!D12=0,'1. Inputs'!D12=""),"-",('1. Inputs'!D53+'1. Inputs'!D54)/'1. Inputs'!D12)</f>
+        <f aca="false">IF(OR('1. Inputs'!D12=0,'1. Inputs'!D12=""),"-",('1. Inputs'!D54+'1. Inputs'!D55)/'1. Inputs'!D12)</f>
         <v>-</v>
       </c>
       <c r="E8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!E12=0,'1. Inputs'!E12=""),"-",('1. Inputs'!E53+'1. Inputs'!E54)/'1. Inputs'!E12)</f>
+        <f aca="false">IF(OR('1. Inputs'!E12=0,'1. Inputs'!E12=""),"-",('1. Inputs'!E54+'1. Inputs'!E55)/'1. Inputs'!E12)</f>
         <v>-</v>
       </c>
       <c r="F8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!F12=0,'1. Inputs'!F12=""),"-",('1. Inputs'!F53+'1. Inputs'!F54)/'1. Inputs'!F12)</f>
+        <f aca="false">IF(OR('1. Inputs'!F12=0,'1. Inputs'!F12=""),"-",('1. Inputs'!F54+'1. Inputs'!F55)/'1. Inputs'!F12)</f>
         <v>-</v>
       </c>
       <c r="G8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!G12=0,'1. Inputs'!G12=""),"-",('1. Inputs'!G53+'1. Inputs'!G54)/'1. Inputs'!G12)</f>
+        <f aca="false">IF(OR('1. Inputs'!G12=0,'1. Inputs'!G12=""),"-",('1. Inputs'!G54+'1. Inputs'!G55)/'1. Inputs'!G12)</f>
         <v>-</v>
       </c>
       <c r="H8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!H12=0,'1. Inputs'!H12=""),"-",('1. Inputs'!H53+'1. Inputs'!H54)/'1. Inputs'!H12)</f>
+        <f aca="false">IF(OR('1. Inputs'!H12=0,'1. Inputs'!H12=""),"-",('1. Inputs'!H54+'1. Inputs'!H55)/'1. Inputs'!H12)</f>
         <v>-</v>
       </c>
       <c r="I8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!I12=0,'1. Inputs'!I12=""),"-",('1. Inputs'!I53+'1. Inputs'!I54)/'1. Inputs'!I12)</f>
+        <f aca="false">IF(OR('1. Inputs'!I12=0,'1. Inputs'!I12=""),"-",('1. Inputs'!I54+'1. Inputs'!I55)/'1. Inputs'!I12)</f>
         <v>-</v>
       </c>
       <c r="J8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!J12=0,'1. Inputs'!J12=""),"-",('1. Inputs'!J53+'1. Inputs'!J54)/'1. Inputs'!J12)</f>
+        <f aca="false">IF(OR('1. Inputs'!J12=0,'1. Inputs'!J12=""),"-",('1. Inputs'!J54+'1. Inputs'!J55)/'1. Inputs'!J12)</f>
         <v>-</v>
       </c>
       <c r="K8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!K12=0,'1. Inputs'!K12=""),"-",('1. Inputs'!K53+'1. Inputs'!K54)/'1. Inputs'!K12)</f>
+        <f aca="false">IF(OR('1. Inputs'!K12=0,'1. Inputs'!K12=""),"-",('1. Inputs'!K54+'1. Inputs'!K55)/'1. Inputs'!K12)</f>
         <v>-</v>
       </c>
       <c r="L8" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!L12=0,'1. Inputs'!L12=""),"-",('1. Inputs'!L53+'1. Inputs'!L54)/'1. Inputs'!L12)</f>
+        <f aca="false">IF(OR('1. Inputs'!L12=0,'1. Inputs'!L12=""),"-",('1. Inputs'!L54+'1. Inputs'!L55)/'1. Inputs'!L12)</f>
         <v>-</v>
       </c>
     </row>
@@ -9091,47 +9326,47 @@
         <v>154</v>
       </c>
       <c r="B9" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!B53+'1. Inputs'!B54)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!B54+'1. Inputs'!B55)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="C9" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!C53+'1. Inputs'!C54)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!C54+'1. Inputs'!C55)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="D9" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!D53+'1. Inputs'!D54)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!D54+'1. Inputs'!D55)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="E9" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!E53+'1. Inputs'!E54)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!E54+'1. Inputs'!E55)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="F9" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!F53+'1. Inputs'!F54)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!F54+'1. Inputs'!F55)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="G9" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!G53+'1. Inputs'!G54)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!G54+'1. Inputs'!G55)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="H9" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!H53+'1. Inputs'!H54)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!H54+'1. Inputs'!H55)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="I9" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!I53+'1. Inputs'!I54)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!I54+'1. Inputs'!I55)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="J9" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!J53+'1. Inputs'!J54)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!J54+'1. Inputs'!J55)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="K9" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!K53+'1. Inputs'!K54)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!K54+'1. Inputs'!K55)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
       <c r="L9" s="11" t="str">
-        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!L53+'1. Inputs'!L54)/'1. Inputs'!$B$5)</f>
+        <f aca="false">IF('1. Inputs'!$B$5=0,"-",('1. Inputs'!L54+'1. Inputs'!L55)/'1. Inputs'!$B$5)</f>
         <v>-</v>
       </c>
     </row>
@@ -9142,45 +9377,45 @@
       <c r="B10" s="12" t="s">
         <v>124</v>
       </c>
-      <c r="C10" s="12" t="e">
-        <f aca="false">IF(('1. Inputs'!B53+'1. Inputs'!B54)=0,"-",(('1. Inputs'!C53+'1. Inputs'!C54)-('1. Inputs'!B53+'1. Inputs'!B54))/ABS('1. Inputs'!B53+'1. Inputs'!B54))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D10" s="12" t="e">
-        <f aca="false">IF(('1. Inputs'!C53+'1. Inputs'!C54)=0,"-",(('1. Inputs'!D53+'1. Inputs'!D54)-('1. Inputs'!C53+'1. Inputs'!C54))/ABS('1. Inputs'!C53+'1. Inputs'!C54))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E10" s="12" t="e">
-        <f aca="false">IF(('1. Inputs'!D53+'1. Inputs'!D54)=0,"-",(('1. Inputs'!E53+'1. Inputs'!E54)-('1. Inputs'!D53+'1. Inputs'!D54))/ABS('1. Inputs'!D53+'1. Inputs'!D54))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F10" s="12" t="e">
-        <f aca="false">IF(('1. Inputs'!E53+'1. Inputs'!E54)=0,"-",(('1. Inputs'!F53+'1. Inputs'!F54)-('1. Inputs'!E53+'1. Inputs'!E54))/ABS('1. Inputs'!E53+'1. Inputs'!E54))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G10" s="12" t="e">
-        <f aca="false">IF(('1. Inputs'!F53+'1. Inputs'!F54)=0,"-",(('1. Inputs'!G53+'1. Inputs'!G54)-('1. Inputs'!F53+'1. Inputs'!F54))/ABS('1. Inputs'!F53+'1. Inputs'!F54))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="H10" s="12" t="e">
-        <f aca="false">IF(('1. Inputs'!G53+'1. Inputs'!G54)=0,"-",(('1. Inputs'!H53+'1. Inputs'!H54)-('1. Inputs'!G53+'1. Inputs'!G54))/ABS('1. Inputs'!G53+'1. Inputs'!G54))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I10" s="12" t="e">
-        <f aca="false">IF(('1. Inputs'!H53+'1. Inputs'!H54)=0,"-",(('1. Inputs'!I53+'1. Inputs'!I54)-('1. Inputs'!H53+'1. Inputs'!H54))/ABS('1. Inputs'!H53+'1. Inputs'!H54))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="J10" s="12" t="e">
-        <f aca="false">IF(('1. Inputs'!I53+'1. Inputs'!I54)=0,"-",(('1. Inputs'!J53+'1. Inputs'!J54)-('1. Inputs'!I53+'1. Inputs'!I54))/ABS('1. Inputs'!I53+'1. Inputs'!I54))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K10" s="12" t="e">
-        <f aca="false">IF(('1. Inputs'!J53+'1. Inputs'!J54)=0,"-",(('1. Inputs'!K53+'1. Inputs'!K54)-('1. Inputs'!J53+'1. Inputs'!J54))/ABS('1. Inputs'!J53+'1. Inputs'!J54))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L10" s="12" t="e">
-        <f aca="false">IF(('1. Inputs'!K53+'1. Inputs'!K54)=0,"-",(('1. Inputs'!L53+'1. Inputs'!L54)-('1. Inputs'!K53+'1. Inputs'!K54))/ABS('1. Inputs'!K53+'1. Inputs'!K54))</f>
-        <v>#VALUE!</v>
+      <c r="C10" s="12" t="str">
+        <f aca="false">IF(('1. Inputs'!B54+'1. Inputs'!B55)=0,"-",(('1. Inputs'!C54+'1. Inputs'!C55)-('1. Inputs'!B54+'1. Inputs'!B55))/ABS('1. Inputs'!B54+'1. Inputs'!B55))</f>
+        <v>-</v>
+      </c>
+      <c r="D10" s="12" t="str">
+        <f aca="false">IF(('1. Inputs'!C54+'1. Inputs'!C55)=0,"-",(('1. Inputs'!D54+'1. Inputs'!D55)-('1. Inputs'!C54+'1. Inputs'!C55))/ABS('1. Inputs'!C54+'1. Inputs'!C55))</f>
+        <v>-</v>
+      </c>
+      <c r="E10" s="12" t="str">
+        <f aca="false">IF(('1. Inputs'!D54+'1. Inputs'!D55)=0,"-",(('1. Inputs'!E54+'1. Inputs'!E55)-('1. Inputs'!D54+'1. Inputs'!D55))/ABS('1. Inputs'!D54+'1. Inputs'!D55))</f>
+        <v>-</v>
+      </c>
+      <c r="F10" s="12" t="str">
+        <f aca="false">IF(('1. Inputs'!E54+'1. Inputs'!E55)=0,"-",(('1. Inputs'!F54+'1. Inputs'!F55)-('1. Inputs'!E54+'1. Inputs'!E55))/ABS('1. Inputs'!E54+'1. Inputs'!E55))</f>
+        <v>-</v>
+      </c>
+      <c r="G10" s="12" t="str">
+        <f aca="false">IF(('1. Inputs'!F54+'1. Inputs'!F55)=0,"-",(('1. Inputs'!G54+'1. Inputs'!G55)-('1. Inputs'!F54+'1. Inputs'!F55))/ABS('1. Inputs'!F54+'1. Inputs'!F55))</f>
+        <v>-</v>
+      </c>
+      <c r="H10" s="12" t="str">
+        <f aca="false">IF(('1. Inputs'!G54+'1. Inputs'!G55)=0,"-",(('1. Inputs'!H54+'1. Inputs'!H55)-('1. Inputs'!G54+'1. Inputs'!G55))/ABS('1. Inputs'!G54+'1. Inputs'!G55))</f>
+        <v>-</v>
+      </c>
+      <c r="I10" s="12" t="str">
+        <f aca="false">IF(('1. Inputs'!H54+'1. Inputs'!H55)=0,"-",(('1. Inputs'!I54+'1. Inputs'!I55)-('1. Inputs'!H54+'1. Inputs'!H55))/ABS('1. Inputs'!H54+'1. Inputs'!H55))</f>
+        <v>-</v>
+      </c>
+      <c r="J10" s="12" t="str">
+        <f aca="false">IF(('1. Inputs'!I54+'1. Inputs'!I55)=0,"-",(('1. Inputs'!J54+'1. Inputs'!J55)-('1. Inputs'!I54+'1. Inputs'!I55))/ABS('1. Inputs'!I54+'1. Inputs'!I55))</f>
+        <v>-</v>
+      </c>
+      <c r="K10" s="12" t="str">
+        <f aca="false">IF(('1. Inputs'!J54+'1. Inputs'!J55)=0,"-",(('1. Inputs'!K54+'1. Inputs'!K55)-('1. Inputs'!J54+'1. Inputs'!J55))/ABS('1. Inputs'!J54+'1. Inputs'!J55))</f>
+        <v>-</v>
+      </c>
+      <c r="L10" s="12" t="str">
+        <f aca="false">IF(('1. Inputs'!K54+'1. Inputs'!K55)=0,"-",(('1. Inputs'!L54+'1. Inputs'!L55)-('1. Inputs'!K54+'1. Inputs'!K55))/ABS('1. Inputs'!K54+'1. Inputs'!K55))</f>
+        <v>-</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9188,47 +9423,47 @@
         <v>156</v>
       </c>
       <c r="B11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!B18=0,'1. Inputs'!B18=""),"-",('1. Inputs'!B53+'1. Inputs'!B54)/'1. Inputs'!B18)</f>
+        <f aca="false">IF(OR('1. Inputs'!B18=0,'1. Inputs'!B18=""),"-",('1. Inputs'!B54+'1. Inputs'!B55)/'1. Inputs'!B18)</f>
         <v>-</v>
       </c>
       <c r="C11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!C18=0,'1. Inputs'!C18=""),"-",('1. Inputs'!C53+'1. Inputs'!C54)/'1. Inputs'!C18)</f>
+        <f aca="false">IF(OR('1. Inputs'!C18=0,'1. Inputs'!C18=""),"-",('1. Inputs'!C54+'1. Inputs'!C55)/'1. Inputs'!C18)</f>
         <v>-</v>
       </c>
       <c r="D11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!D18=0,'1. Inputs'!D18=""),"-",('1. Inputs'!D53+'1. Inputs'!D54)/'1. Inputs'!D18)</f>
+        <f aca="false">IF(OR('1. Inputs'!D18=0,'1. Inputs'!D18=""),"-",('1. Inputs'!D54+'1. Inputs'!D55)/'1. Inputs'!D18)</f>
         <v>-</v>
       </c>
       <c r="E11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!E18=0,'1. Inputs'!E18=""),"-",('1. Inputs'!E53+'1. Inputs'!E54)/'1. Inputs'!E18)</f>
+        <f aca="false">IF(OR('1. Inputs'!E18=0,'1. Inputs'!E18=""),"-",('1. Inputs'!E54+'1. Inputs'!E55)/'1. Inputs'!E18)</f>
         <v>-</v>
       </c>
       <c r="F11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!F18=0,'1. Inputs'!F18=""),"-",('1. Inputs'!F53+'1. Inputs'!F54)/'1. Inputs'!F18)</f>
+        <f aca="false">IF(OR('1. Inputs'!F18=0,'1. Inputs'!F18=""),"-",('1. Inputs'!F54+'1. Inputs'!F55)/'1. Inputs'!F18)</f>
         <v>-</v>
       </c>
       <c r="G11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!G18=0,'1. Inputs'!G18=""),"-",('1. Inputs'!G53+'1. Inputs'!G54)/'1. Inputs'!G18)</f>
+        <f aca="false">IF(OR('1. Inputs'!G18=0,'1. Inputs'!G18=""),"-",('1. Inputs'!G54+'1. Inputs'!G55)/'1. Inputs'!G18)</f>
         <v>-</v>
       </c>
       <c r="H11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!H18=0,'1. Inputs'!H18=""),"-",('1. Inputs'!H53+'1. Inputs'!H54)/'1. Inputs'!H18)</f>
+        <f aca="false">IF(OR('1. Inputs'!H18=0,'1. Inputs'!H18=""),"-",('1. Inputs'!H54+'1. Inputs'!H55)/'1. Inputs'!H18)</f>
         <v>-</v>
       </c>
       <c r="I11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!I18=0,'1. Inputs'!I18=""),"-",('1. Inputs'!I53+'1. Inputs'!I54)/'1. Inputs'!I18)</f>
+        <f aca="false">IF(OR('1. Inputs'!I18=0,'1. Inputs'!I18=""),"-",('1. Inputs'!I54+'1. Inputs'!I55)/'1. Inputs'!I18)</f>
         <v>-</v>
       </c>
       <c r="J11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!J18=0,'1. Inputs'!J18=""),"-",('1. Inputs'!J53+'1. Inputs'!J54)/'1. Inputs'!J18)</f>
+        <f aca="false">IF(OR('1. Inputs'!J18=0,'1. Inputs'!J18=""),"-",('1. Inputs'!J54+'1. Inputs'!J55)/'1. Inputs'!J18)</f>
         <v>-</v>
       </c>
       <c r="K11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!K18=0,'1. Inputs'!K18=""),"-",('1. Inputs'!K53+'1. Inputs'!K54)/'1. Inputs'!K18)</f>
+        <f aca="false">IF(OR('1. Inputs'!K18=0,'1. Inputs'!K18=""),"-",('1. Inputs'!K54+'1. Inputs'!K55)/'1. Inputs'!K18)</f>
         <v>-</v>
       </c>
       <c r="L11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!L18=0,'1. Inputs'!L18=""),"-",('1. Inputs'!L53+'1. Inputs'!L54)/'1. Inputs'!L18)</f>
+        <f aca="false">IF(OR('1. Inputs'!L18=0,'1. Inputs'!L18=""),"-",('1. Inputs'!L54+'1. Inputs'!L55)/'1. Inputs'!L18)</f>
         <v>-</v>
       </c>
     </row>
@@ -9237,47 +9472,47 @@
         <v>157</v>
       </c>
       <c r="B12" s="11" t="n">
-        <f aca="false">'1. Inputs'!B57</f>
+        <f aca="false">'1. Inputs'!B58</f>
         <v>0</v>
       </c>
       <c r="C12" s="11" t="n">
-        <f aca="false">'1. Inputs'!C57</f>
+        <f aca="false">'1. Inputs'!C58</f>
         <v>0</v>
       </c>
       <c r="D12" s="11" t="n">
-        <f aca="false">'1. Inputs'!D57</f>
+        <f aca="false">'1. Inputs'!D58</f>
         <v>0</v>
       </c>
       <c r="E12" s="11" t="n">
-        <f aca="false">'1. Inputs'!E57</f>
+        <f aca="false">'1. Inputs'!E58</f>
         <v>0</v>
       </c>
       <c r="F12" s="11" t="n">
-        <f aca="false">'1. Inputs'!F57</f>
+        <f aca="false">'1. Inputs'!F58</f>
         <v>0</v>
       </c>
       <c r="G12" s="11" t="n">
-        <f aca="false">'1. Inputs'!G57</f>
+        <f aca="false">'1. Inputs'!G58</f>
         <v>0</v>
       </c>
       <c r="H12" s="11" t="n">
-        <f aca="false">'1. Inputs'!H57</f>
+        <f aca="false">'1. Inputs'!H58</f>
         <v>0</v>
       </c>
       <c r="I12" s="11" t="n">
-        <f aca="false">'1. Inputs'!I57</f>
+        <f aca="false">'1. Inputs'!I58</f>
         <v>0</v>
       </c>
       <c r="J12" s="11" t="n">
-        <f aca="false">'1. Inputs'!J57</f>
+        <f aca="false">'1. Inputs'!J58</f>
         <v>0</v>
       </c>
       <c r="K12" s="11" t="n">
-        <f aca="false">'1. Inputs'!K57</f>
+        <f aca="false">'1. Inputs'!K58</f>
         <v>0</v>
       </c>
       <c r="L12" s="11" t="n">
-        <f aca="false">'1. Inputs'!L57</f>
+        <f aca="false">'1. Inputs'!L58</f>
         <v>0</v>
       </c>
     </row>
@@ -9286,47 +9521,47 @@
         <v>158</v>
       </c>
       <c r="B13" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!B18=0,'1. Inputs'!B18=""),"-",'1. Inputs'!B57/'1. Inputs'!B18)</f>
+        <f aca="false">IF(OR('1. Inputs'!B18=0,'1. Inputs'!B18=""),"-",'1. Inputs'!B58/'1. Inputs'!B18)</f>
         <v>-</v>
       </c>
       <c r="C13" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!C18=0,'1. Inputs'!C18=""),"-",'1. Inputs'!C57/'1. Inputs'!C18)</f>
+        <f aca="false">IF(OR('1. Inputs'!C18=0,'1. Inputs'!C18=""),"-",'1. Inputs'!C58/'1. Inputs'!C18)</f>
         <v>-</v>
       </c>
       <c r="D13" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!D18=0,'1. Inputs'!D18=""),"-",'1. Inputs'!D57/'1. Inputs'!D18)</f>
+        <f aca="false">IF(OR('1. Inputs'!D18=0,'1. Inputs'!D18=""),"-",'1. Inputs'!D58/'1. Inputs'!D18)</f>
         <v>-</v>
       </c>
       <c r="E13" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!E18=0,'1. Inputs'!E18=""),"-",'1. Inputs'!E57/'1. Inputs'!E18)</f>
+        <f aca="false">IF(OR('1. Inputs'!E18=0,'1. Inputs'!E18=""),"-",'1. Inputs'!E58/'1. Inputs'!E18)</f>
         <v>-</v>
       </c>
       <c r="F13" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!F18=0,'1. Inputs'!F18=""),"-",'1. Inputs'!F57/'1. Inputs'!F18)</f>
+        <f aca="false">IF(OR('1. Inputs'!F18=0,'1. Inputs'!F18=""),"-",'1. Inputs'!F58/'1. Inputs'!F18)</f>
         <v>-</v>
       </c>
       <c r="G13" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!G18=0,'1. Inputs'!G18=""),"-",'1. Inputs'!G57/'1. Inputs'!G18)</f>
+        <f aca="false">IF(OR('1. Inputs'!G18=0,'1. Inputs'!G18=""),"-",'1. Inputs'!G58/'1. Inputs'!G18)</f>
         <v>-</v>
       </c>
       <c r="H13" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!H18=0,'1. Inputs'!H18=""),"-",'1. Inputs'!H57/'1. Inputs'!H18)</f>
+        <f aca="false">IF(OR('1. Inputs'!H18=0,'1. Inputs'!H18=""),"-",'1. Inputs'!H58/'1. Inputs'!H18)</f>
         <v>-</v>
       </c>
       <c r="I13" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!I18=0,'1. Inputs'!I18=""),"-",'1. Inputs'!I57/'1. Inputs'!I18)</f>
+        <f aca="false">IF(OR('1. Inputs'!I18=0,'1. Inputs'!I18=""),"-",'1. Inputs'!I58/'1. Inputs'!I18)</f>
         <v>-</v>
       </c>
       <c r="J13" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!J18=0,'1. Inputs'!J18=""),"-",'1. Inputs'!J57/'1. Inputs'!J18)</f>
+        <f aca="false">IF(OR('1. Inputs'!J18=0,'1. Inputs'!J18=""),"-",'1. Inputs'!J58/'1. Inputs'!J18)</f>
         <v>-</v>
       </c>
       <c r="K13" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!K18=0,'1. Inputs'!K18=""),"-",'1. Inputs'!K57/'1. Inputs'!K18)</f>
+        <f aca="false">IF(OR('1. Inputs'!K18=0,'1. Inputs'!K18=""),"-",'1. Inputs'!K58/'1. Inputs'!K18)</f>
         <v>-</v>
       </c>
       <c r="L13" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!L18=0,'1. Inputs'!L18=""),"-",'1. Inputs'!L57/'1. Inputs'!L18)</f>
+        <f aca="false">IF(OR('1. Inputs'!L18=0,'1. Inputs'!L18=""),"-",'1. Inputs'!L58/'1. Inputs'!L18)</f>
         <v>-</v>
       </c>
     </row>
@@ -9335,47 +9570,47 @@
         <v>100</v>
       </c>
       <c r="B14" s="11" t="n">
-        <f aca="false">'1. Inputs'!B59</f>
+        <f aca="false">'1. Inputs'!B60</f>
         <v>0</v>
       </c>
       <c r="C14" s="11" t="n">
-        <f aca="false">'1. Inputs'!C59</f>
+        <f aca="false">'1. Inputs'!C60</f>
         <v>0</v>
       </c>
       <c r="D14" s="11" t="n">
-        <f aca="false">'1. Inputs'!D59</f>
+        <f aca="false">'1. Inputs'!D60</f>
         <v>0</v>
       </c>
       <c r="E14" s="11" t="n">
-        <f aca="false">'1. Inputs'!E59</f>
+        <f aca="false">'1. Inputs'!E60</f>
         <v>0</v>
       </c>
       <c r="F14" s="11" t="n">
-        <f aca="false">'1. Inputs'!F59</f>
+        <f aca="false">'1. Inputs'!F60</f>
         <v>0</v>
       </c>
       <c r="G14" s="11" t="n">
-        <f aca="false">'1. Inputs'!G59</f>
+        <f aca="false">'1. Inputs'!G60</f>
         <v>0</v>
       </c>
       <c r="H14" s="11" t="n">
-        <f aca="false">'1. Inputs'!H59</f>
+        <f aca="false">'1. Inputs'!H60</f>
         <v>0</v>
       </c>
       <c r="I14" s="11" t="n">
-        <f aca="false">'1. Inputs'!I59</f>
+        <f aca="false">'1. Inputs'!I60</f>
         <v>0</v>
       </c>
       <c r="J14" s="11" t="n">
-        <f aca="false">'1. Inputs'!J59</f>
+        <f aca="false">'1. Inputs'!J60</f>
         <v>0</v>
       </c>
       <c r="K14" s="11" t="n">
-        <f aca="false">'1. Inputs'!K59</f>
+        <f aca="false">'1. Inputs'!K60</f>
         <v>0</v>
       </c>
       <c r="L14" s="11" t="n">
-        <f aca="false">'1. Inputs'!L59</f>
+        <f aca="false">'1. Inputs'!L60</f>
         <v>0</v>
       </c>
     </row>
@@ -9384,47 +9619,47 @@
         <v>159</v>
       </c>
       <c r="B15" s="11" t="n">
-        <f aca="false">'1. Inputs'!B18-ABS('1. Inputs'!B59)</f>
+        <f aca="false">'1. Inputs'!B18-ABS('1. Inputs'!B60)</f>
         <v>0</v>
       </c>
       <c r="C15" s="11" t="n">
-        <f aca="false">'1. Inputs'!C18-ABS('1. Inputs'!C59)</f>
+        <f aca="false">'1. Inputs'!C18-ABS('1. Inputs'!C60)</f>
         <v>0</v>
       </c>
       <c r="D15" s="11" t="n">
-        <f aca="false">'1. Inputs'!D18-ABS('1. Inputs'!D59)</f>
+        <f aca="false">'1. Inputs'!D18-ABS('1. Inputs'!D60)</f>
         <v>0</v>
       </c>
       <c r="E15" s="11" t="n">
-        <f aca="false">'1. Inputs'!E18-ABS('1. Inputs'!E59)</f>
+        <f aca="false">'1. Inputs'!E18-ABS('1. Inputs'!E60)</f>
         <v>0</v>
       </c>
       <c r="F15" s="11" t="n">
-        <f aca="false">'1. Inputs'!F18-ABS('1. Inputs'!F59)</f>
+        <f aca="false">'1. Inputs'!F18-ABS('1. Inputs'!F60)</f>
         <v>0</v>
       </c>
       <c r="G15" s="11" t="n">
-        <f aca="false">'1. Inputs'!G18-ABS('1. Inputs'!G59)</f>
+        <f aca="false">'1. Inputs'!G18-ABS('1. Inputs'!G60)</f>
         <v>0</v>
       </c>
       <c r="H15" s="11" t="n">
-        <f aca="false">'1. Inputs'!H18-ABS('1. Inputs'!H59)</f>
+        <f aca="false">'1. Inputs'!H18-ABS('1. Inputs'!H60)</f>
         <v>0</v>
       </c>
       <c r="I15" s="11" t="n">
-        <f aca="false">'1. Inputs'!I18-ABS('1. Inputs'!I59)</f>
+        <f aca="false">'1. Inputs'!I18-ABS('1. Inputs'!I60)</f>
         <v>0</v>
       </c>
       <c r="J15" s="11" t="n">
-        <f aca="false">'1. Inputs'!J18-ABS('1. Inputs'!J59)</f>
+        <f aca="false">'1. Inputs'!J18-ABS('1. Inputs'!J60)</f>
         <v>0</v>
       </c>
       <c r="K15" s="11" t="n">
-        <f aca="false">'1. Inputs'!K18-ABS('1. Inputs'!K59)</f>
+        <f aca="false">'1. Inputs'!K18-ABS('1. Inputs'!K60)</f>
         <v>0</v>
       </c>
       <c r="L15" s="11" t="n">
-        <f aca="false">'1. Inputs'!L18-ABS('1. Inputs'!L59)</f>
+        <f aca="false">'1. Inputs'!L18-ABS('1. Inputs'!L60)</f>
         <v>0</v>
       </c>
     </row>
@@ -9433,47 +9668,47 @@
         <v>160</v>
       </c>
       <c r="B16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!B18=0,'1. Inputs'!B18=""),"-",1-ABS('1. Inputs'!B59)/'1. Inputs'!B18)</f>
+        <f aca="false">IF(OR('1. Inputs'!B18=0,'1. Inputs'!B18=""),"-",1-ABS('1. Inputs'!B60)/'1. Inputs'!B18)</f>
         <v>-</v>
       </c>
       <c r="C16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!C18=0,'1. Inputs'!C18=""),"-",1-ABS('1. Inputs'!C59)/'1. Inputs'!C18)</f>
+        <f aca="false">IF(OR('1. Inputs'!C18=0,'1. Inputs'!C18=""),"-",1-ABS('1. Inputs'!C60)/'1. Inputs'!C18)</f>
         <v>-</v>
       </c>
       <c r="D16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!D18=0,'1. Inputs'!D18=""),"-",1-ABS('1. Inputs'!D59)/'1. Inputs'!D18)</f>
+        <f aca="false">IF(OR('1. Inputs'!D18=0,'1. Inputs'!D18=""),"-",1-ABS('1. Inputs'!D60)/'1. Inputs'!D18)</f>
         <v>-</v>
       </c>
       <c r="E16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!E18=0,'1. Inputs'!E18=""),"-",1-ABS('1. Inputs'!E59)/'1. Inputs'!E18)</f>
+        <f aca="false">IF(OR('1. Inputs'!E18=0,'1. Inputs'!E18=""),"-",1-ABS('1. Inputs'!E60)/'1. Inputs'!E18)</f>
         <v>-</v>
       </c>
       <c r="F16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!F18=0,'1. Inputs'!F18=""),"-",1-ABS('1. Inputs'!F59)/'1. Inputs'!F18)</f>
+        <f aca="false">IF(OR('1. Inputs'!F18=0,'1. Inputs'!F18=""),"-",1-ABS('1. Inputs'!F60)/'1. Inputs'!F18)</f>
         <v>-</v>
       </c>
       <c r="G16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!G18=0,'1. Inputs'!G18=""),"-",1-ABS('1. Inputs'!G59)/'1. Inputs'!G18)</f>
+        <f aca="false">IF(OR('1. Inputs'!G18=0,'1. Inputs'!G18=""),"-",1-ABS('1. Inputs'!G60)/'1. Inputs'!G18)</f>
         <v>-</v>
       </c>
       <c r="H16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!H18=0,'1. Inputs'!H18=""),"-",1-ABS('1. Inputs'!H59)/'1. Inputs'!H18)</f>
+        <f aca="false">IF(OR('1. Inputs'!H18=0,'1. Inputs'!H18=""),"-",1-ABS('1. Inputs'!H60)/'1. Inputs'!H18)</f>
         <v>-</v>
       </c>
       <c r="I16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!I18=0,'1. Inputs'!I18=""),"-",1-ABS('1. Inputs'!I59)/'1. Inputs'!I18)</f>
+        <f aca="false">IF(OR('1. Inputs'!I18=0,'1. Inputs'!I18=""),"-",1-ABS('1. Inputs'!I60)/'1. Inputs'!I18)</f>
         <v>-</v>
       </c>
       <c r="J16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!J18=0,'1. Inputs'!J18=""),"-",1-ABS('1. Inputs'!J59)/'1. Inputs'!J18)</f>
+        <f aca="false">IF(OR('1. Inputs'!J18=0,'1. Inputs'!J18=""),"-",1-ABS('1. Inputs'!J60)/'1. Inputs'!J18)</f>
         <v>-</v>
       </c>
       <c r="K16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!K18=0,'1. Inputs'!K18=""),"-",1-ABS('1. Inputs'!K59)/'1. Inputs'!K18)</f>
+        <f aca="false">IF(OR('1. Inputs'!K18=0,'1. Inputs'!K18=""),"-",1-ABS('1. Inputs'!K60)/'1. Inputs'!K18)</f>
         <v>-</v>
       </c>
       <c r="L16" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!L18=0,'1. Inputs'!L18=""),"-",1-ABS('1. Inputs'!L59)/'1. Inputs'!L18)</f>
+        <f aca="false">IF(OR('1. Inputs'!L18=0,'1. Inputs'!L18=""),"-",1-ABS('1. Inputs'!L60)/'1. Inputs'!L18)</f>
         <v>-</v>
       </c>
     </row>
@@ -9573,47 +9808,47 @@
         <v>162</v>
       </c>
       <c r="B4" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!B33=0,'1. Inputs'!B33=""),"-",'1. Inputs'!B18/'1. Inputs'!B33)</f>
+        <f aca="false">IF(OR('1. Inputs'!B34=0,'1. Inputs'!B34=""),"-",'1. Inputs'!B18/'1. Inputs'!B34)</f>
         <v>-</v>
       </c>
       <c r="C4" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!C33+'1. Inputs'!B33)/2=0),"-",'1. Inputs'!C18/(('1. Inputs'!C33+'1. Inputs'!B33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!C34+'1. Inputs'!B34)/2=0),"-",'1. Inputs'!C18/(('1. Inputs'!C34+'1. Inputs'!B34)/2))</f>
         <v>-</v>
       </c>
       <c r="D4" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!D33+'1. Inputs'!C33)/2=0),"-",'1. Inputs'!D18/(('1. Inputs'!D33+'1. Inputs'!C33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!D34+'1. Inputs'!C34)/2=0),"-",'1. Inputs'!D18/(('1. Inputs'!D34+'1. Inputs'!C34)/2))</f>
         <v>-</v>
       </c>
       <c r="E4" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!E33+'1. Inputs'!D33)/2=0),"-",'1. Inputs'!E18/(('1. Inputs'!E33+'1. Inputs'!D33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!E34+'1. Inputs'!D34)/2=0),"-",'1. Inputs'!E18/(('1. Inputs'!E34+'1. Inputs'!D34)/2))</f>
         <v>-</v>
       </c>
       <c r="F4" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!F33+'1. Inputs'!E33)/2=0),"-",'1. Inputs'!F18/(('1. Inputs'!F33+'1. Inputs'!E33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!F34+'1. Inputs'!E34)/2=0),"-",'1. Inputs'!F18/(('1. Inputs'!F34+'1. Inputs'!E34)/2))</f>
         <v>-</v>
       </c>
       <c r="G4" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!G33+'1. Inputs'!F33)/2=0),"-",'1. Inputs'!G18/(('1. Inputs'!G33+'1. Inputs'!F33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!G34+'1. Inputs'!F34)/2=0),"-",'1. Inputs'!G18/(('1. Inputs'!G34+'1. Inputs'!F34)/2))</f>
         <v>-</v>
       </c>
       <c r="H4" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!H33+'1. Inputs'!G33)/2=0),"-",'1. Inputs'!H18/(('1. Inputs'!H33+'1. Inputs'!G33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!H34+'1. Inputs'!G34)/2=0),"-",'1. Inputs'!H18/(('1. Inputs'!H34+'1. Inputs'!G34)/2))</f>
         <v>-</v>
       </c>
       <c r="I4" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!I33+'1. Inputs'!H33)/2=0),"-",'1. Inputs'!I18/(('1. Inputs'!I33+'1. Inputs'!H33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!I34+'1. Inputs'!H34)/2=0),"-",'1. Inputs'!I18/(('1. Inputs'!I34+'1. Inputs'!H34)/2))</f>
         <v>-</v>
       </c>
       <c r="J4" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!J33+'1. Inputs'!I33)/2=0),"-",'1. Inputs'!J18/(('1. Inputs'!J33+'1. Inputs'!I33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!J34+'1. Inputs'!I34)/2=0),"-",'1. Inputs'!J18/(('1. Inputs'!J34+'1. Inputs'!I34)/2))</f>
         <v>-</v>
       </c>
       <c r="K4" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!K33+'1. Inputs'!J33)/2=0),"-",'1. Inputs'!K18/(('1. Inputs'!K33+'1. Inputs'!J33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!K34+'1. Inputs'!J34)/2=0),"-",'1. Inputs'!K18/(('1. Inputs'!K34+'1. Inputs'!J34)/2))</f>
         <v>-</v>
       </c>
       <c r="L4" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!L33+'1. Inputs'!K33)/2=0),"-",'1. Inputs'!L18/(('1. Inputs'!L33+'1. Inputs'!K33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!L34+'1. Inputs'!K34)/2=0),"-",'1. Inputs'!L18/(('1. Inputs'!L34+'1. Inputs'!K34)/2))</f>
         <v>-</v>
       </c>
     </row>
@@ -9621,49 +9856,49 @@
       <c r="A5" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="B5" s="12" t="e">
-        <f aca="false">IF(OR('1. Inputs'!B31=0,'1. Inputs'!B31=""),"-",'1. Inputs'!B18/'1. Inputs'!B31)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C5" s="12" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!C31+'1. Inputs'!B31)/2=0),"-",'1. Inputs'!C18/(('1. Inputs'!C31+'1. Inputs'!B31)/2))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D5" s="12" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!D31+'1. Inputs'!C31)/2=0),"-",'1. Inputs'!D18/(('1. Inputs'!D31+'1. Inputs'!C31)/2))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E5" s="12" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!E31+'1. Inputs'!D31)/2=0),"-",'1. Inputs'!E18/(('1. Inputs'!E31+'1. Inputs'!D31)/2))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F5" s="12" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!F31+'1. Inputs'!E31)/2=0),"-",'1. Inputs'!F18/(('1. Inputs'!F31+'1. Inputs'!E31)/2))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G5" s="12" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!G31+'1. Inputs'!F31)/2=0),"-",'1. Inputs'!G18/(('1. Inputs'!G31+'1. Inputs'!F31)/2))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="H5" s="12" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!H31+'1. Inputs'!G31)/2=0),"-",'1. Inputs'!H18/(('1. Inputs'!H31+'1. Inputs'!G31)/2))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I5" s="12" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!I31+'1. Inputs'!H31)/2=0),"-",'1. Inputs'!I18/(('1. Inputs'!I31+'1. Inputs'!H31)/2))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="J5" s="12" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!J31+'1. Inputs'!I31)/2=0),"-",'1. Inputs'!J18/(('1. Inputs'!J31+'1. Inputs'!I31)/2))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K5" s="12" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!K31+'1. Inputs'!J31)/2=0),"-",'1. Inputs'!K18/(('1. Inputs'!K31+'1. Inputs'!J31)/2))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L5" s="12" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!L31+'1. Inputs'!K31)/2=0),"-",'1. Inputs'!L18/(('1. Inputs'!L31+'1. Inputs'!K31)/2))</f>
-        <v>#VALUE!</v>
+      <c r="B5" s="12" t="str">
+        <f aca="false">IF(OR('1. Inputs'!B32=0,'1. Inputs'!B32=""),"-",'1. Inputs'!B18/'1. Inputs'!B32)</f>
+        <v>-</v>
+      </c>
+      <c r="C5" s="12" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!C32+'1. Inputs'!B32)/2=0),"-",'1. Inputs'!C18/(('1. Inputs'!C32+'1. Inputs'!B32)/2))</f>
+        <v>-</v>
+      </c>
+      <c r="D5" s="12" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!D32+'1. Inputs'!C32)/2=0),"-",'1. Inputs'!D18/(('1. Inputs'!D32+'1. Inputs'!C32)/2))</f>
+        <v>-</v>
+      </c>
+      <c r="E5" s="12" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!E32+'1. Inputs'!D32)/2=0),"-",'1. Inputs'!E18/(('1. Inputs'!E32+'1. Inputs'!D32)/2))</f>
+        <v>-</v>
+      </c>
+      <c r="F5" s="12" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!F32+'1. Inputs'!E32)/2=0),"-",'1. Inputs'!F18/(('1. Inputs'!F32+'1. Inputs'!E32)/2))</f>
+        <v>-</v>
+      </c>
+      <c r="G5" s="12" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!G32+'1. Inputs'!F32)/2=0),"-",'1. Inputs'!G18/(('1. Inputs'!G32+'1. Inputs'!F32)/2))</f>
+        <v>-</v>
+      </c>
+      <c r="H5" s="12" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!H32+'1. Inputs'!G32)/2=0),"-",'1. Inputs'!H18/(('1. Inputs'!H32+'1. Inputs'!G32)/2))</f>
+        <v>-</v>
+      </c>
+      <c r="I5" s="12" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!I32+'1. Inputs'!H32)/2=0),"-",'1. Inputs'!I18/(('1. Inputs'!I32+'1. Inputs'!H32)/2))</f>
+        <v>-</v>
+      </c>
+      <c r="J5" s="12" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!J32+'1. Inputs'!I32)/2=0),"-",'1. Inputs'!J18/(('1. Inputs'!J32+'1. Inputs'!I32)/2))</f>
+        <v>-</v>
+      </c>
+      <c r="K5" s="12" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!K32+'1. Inputs'!J32)/2=0),"-",'1. Inputs'!K18/(('1. Inputs'!K32+'1. Inputs'!J32)/2))</f>
+        <v>-</v>
+      </c>
+      <c r="L5" s="12" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!L32+'1. Inputs'!K32)/2=0),"-",'1. Inputs'!L18/(('1. Inputs'!L32+'1. Inputs'!K32)/2))</f>
+        <v>-</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9724,49 +9959,49 @@
       <c r="A8" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="B8" s="14" t="e">
-        <f aca="false">IF(OR('1. Inputs'!B31=0),"-",'1. Inputs'!B12/'1. Inputs'!B31)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C8" s="14" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!C31+'1. Inputs'!B31)/2=0),"-",'1. Inputs'!C12/(('1. Inputs'!C31+'1. Inputs'!B31)/2))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D8" s="14" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!D31+'1. Inputs'!C31)/2=0),"-",'1. Inputs'!D12/(('1. Inputs'!D31+'1. Inputs'!C31)/2))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E8" s="14" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!E31+'1. Inputs'!D31)/2=0),"-",'1. Inputs'!E12/(('1. Inputs'!E31+'1. Inputs'!D31)/2))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F8" s="14" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!F31+'1. Inputs'!E31)/2=0),"-",'1. Inputs'!F12/(('1. Inputs'!F31+'1. Inputs'!E31)/2))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G8" s="14" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!G31+'1. Inputs'!F31)/2=0),"-",'1. Inputs'!G12/(('1. Inputs'!G31+'1. Inputs'!F31)/2))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="H8" s="14" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!H31+'1. Inputs'!G31)/2=0),"-",'1. Inputs'!H12/(('1. Inputs'!H31+'1. Inputs'!G31)/2))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I8" s="14" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!I31+'1. Inputs'!H31)/2=0),"-",'1. Inputs'!I12/(('1. Inputs'!I31+'1. Inputs'!H31)/2))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="J8" s="14" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!J31+'1. Inputs'!I31)/2=0),"-",'1. Inputs'!J12/(('1. Inputs'!J31+'1. Inputs'!I31)/2))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K8" s="14" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!K31+'1. Inputs'!J31)/2=0),"-",'1. Inputs'!K12/(('1. Inputs'!K31+'1. Inputs'!J31)/2))</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L8" s="14" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!L31+'1. Inputs'!K31)/2=0),"-",'1. Inputs'!L12/(('1. Inputs'!L31+'1. Inputs'!K31)/2))</f>
-        <v>#VALUE!</v>
+      <c r="B8" s="14" t="str">
+        <f aca="false">IF(OR('1. Inputs'!B32=0),"-",'1. Inputs'!B12/'1. Inputs'!B32)</f>
+        <v>-</v>
+      </c>
+      <c r="C8" s="14" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!C32+'1. Inputs'!B32)/2=0),"-",'1. Inputs'!C12/(('1. Inputs'!C32+'1. Inputs'!B32)/2))</f>
+        <v>-</v>
+      </c>
+      <c r="D8" s="14" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!D32+'1. Inputs'!C32)/2=0),"-",'1. Inputs'!D12/(('1. Inputs'!D32+'1. Inputs'!C32)/2))</f>
+        <v>-</v>
+      </c>
+      <c r="E8" s="14" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!E32+'1. Inputs'!D32)/2=0),"-",'1. Inputs'!E12/(('1. Inputs'!E32+'1. Inputs'!D32)/2))</f>
+        <v>-</v>
+      </c>
+      <c r="F8" s="14" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!F32+'1. Inputs'!E32)/2=0),"-",'1. Inputs'!F12/(('1. Inputs'!F32+'1. Inputs'!E32)/2))</f>
+        <v>-</v>
+      </c>
+      <c r="G8" s="14" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!G32+'1. Inputs'!F32)/2=0),"-",'1. Inputs'!G12/(('1. Inputs'!G32+'1. Inputs'!F32)/2))</f>
+        <v>-</v>
+      </c>
+      <c r="H8" s="14" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!H32+'1. Inputs'!G32)/2=0),"-",'1. Inputs'!H12/(('1. Inputs'!H32+'1. Inputs'!G32)/2))</f>
+        <v>-</v>
+      </c>
+      <c r="I8" s="14" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!I32+'1. Inputs'!H32)/2=0),"-",'1. Inputs'!I12/(('1. Inputs'!I32+'1. Inputs'!H32)/2))</f>
+        <v>-</v>
+      </c>
+      <c r="J8" s="14" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!J32+'1. Inputs'!I32)/2=0),"-",'1. Inputs'!J12/(('1. Inputs'!J32+'1. Inputs'!I32)/2))</f>
+        <v>-</v>
+      </c>
+      <c r="K8" s="14" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!K32+'1. Inputs'!J32)/2=0),"-",'1. Inputs'!K12/(('1. Inputs'!K32+'1. Inputs'!J32)/2))</f>
+        <v>-</v>
+      </c>
+      <c r="L8" s="14" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!L32+'1. Inputs'!K32)/2=0),"-",'1. Inputs'!L12/(('1. Inputs'!L32+'1. Inputs'!K32)/2))</f>
+        <v>-</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9774,47 +10009,47 @@
         <v>167</v>
       </c>
       <c r="B9" s="14" t="str">
-        <f aca="false">IF(OR('1. Inputs'!B33=0),"-",'1. Inputs'!B31/'1. Inputs'!B33)</f>
+        <f aca="false">IF(OR('1. Inputs'!B34=0),"-",'1. Inputs'!B32/'1. Inputs'!B34)</f>
         <v>-</v>
       </c>
       <c r="C9" s="14" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!C33+'1. Inputs'!B33)/2=0),"-",(('1. Inputs'!C31+'1. Inputs'!B31)/2)/(('1. Inputs'!C33+'1. Inputs'!B33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!C34+'1. Inputs'!B34)/2=0),"-",(('1. Inputs'!C32+'1. Inputs'!B32)/2)/(('1. Inputs'!C34+'1. Inputs'!B34)/2))</f>
         <v>-</v>
       </c>
       <c r="D9" s="14" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!D33+'1. Inputs'!C33)/2=0),"-",(('1. Inputs'!D31+'1. Inputs'!C31)/2)/(('1. Inputs'!D33+'1. Inputs'!C33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!D34+'1. Inputs'!C34)/2=0),"-",(('1. Inputs'!D32+'1. Inputs'!C32)/2)/(('1. Inputs'!D34+'1. Inputs'!C34)/2))</f>
         <v>-</v>
       </c>
       <c r="E9" s="14" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!E33+'1. Inputs'!D33)/2=0),"-",(('1. Inputs'!E31+'1. Inputs'!D31)/2)/(('1. Inputs'!E33+'1. Inputs'!D33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!E34+'1. Inputs'!D34)/2=0),"-",(('1. Inputs'!E32+'1. Inputs'!D32)/2)/(('1. Inputs'!E34+'1. Inputs'!D34)/2))</f>
         <v>-</v>
       </c>
       <c r="F9" s="14" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!F33+'1. Inputs'!E33)/2=0),"-",(('1. Inputs'!F31+'1. Inputs'!E31)/2)/(('1. Inputs'!F33+'1. Inputs'!E33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!F34+'1. Inputs'!E34)/2=0),"-",(('1. Inputs'!F32+'1. Inputs'!E32)/2)/(('1. Inputs'!F34+'1. Inputs'!E34)/2))</f>
         <v>-</v>
       </c>
       <c r="G9" s="14" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!G33+'1. Inputs'!F33)/2=0),"-",(('1. Inputs'!G31+'1. Inputs'!F31)/2)/(('1. Inputs'!G33+'1. Inputs'!F33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!G34+'1. Inputs'!F34)/2=0),"-",(('1. Inputs'!G32+'1. Inputs'!F32)/2)/(('1. Inputs'!G34+'1. Inputs'!F34)/2))</f>
         <v>-</v>
       </c>
       <c r="H9" s="14" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!H33+'1. Inputs'!G33)/2=0),"-",(('1. Inputs'!H31+'1. Inputs'!G31)/2)/(('1. Inputs'!H33+'1. Inputs'!G33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!H34+'1. Inputs'!G34)/2=0),"-",(('1. Inputs'!H32+'1. Inputs'!G32)/2)/(('1. Inputs'!H34+'1. Inputs'!G34)/2))</f>
         <v>-</v>
       </c>
       <c r="I9" s="14" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!I33+'1. Inputs'!H33)/2=0),"-",(('1. Inputs'!I31+'1. Inputs'!H31)/2)/(('1. Inputs'!I33+'1. Inputs'!H33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!I34+'1. Inputs'!H34)/2=0),"-",(('1. Inputs'!I32+'1. Inputs'!H32)/2)/(('1. Inputs'!I34+'1. Inputs'!H34)/2))</f>
         <v>-</v>
       </c>
       <c r="J9" s="14" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!J33+'1. Inputs'!I33)/2=0),"-",(('1. Inputs'!J31+'1. Inputs'!I31)/2)/(('1. Inputs'!J33+'1. Inputs'!I33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!J34+'1. Inputs'!I34)/2=0),"-",(('1. Inputs'!J32+'1. Inputs'!I32)/2)/(('1. Inputs'!J34+'1. Inputs'!I34)/2))</f>
         <v>-</v>
       </c>
       <c r="K9" s="14" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!K33+'1. Inputs'!J33)/2=0),"-",(('1. Inputs'!K31+'1. Inputs'!J31)/2)/(('1. Inputs'!K33+'1. Inputs'!J33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!K34+'1. Inputs'!J34)/2=0),"-",(('1. Inputs'!K32+'1. Inputs'!J32)/2)/(('1. Inputs'!K34+'1. Inputs'!J34)/2))</f>
         <v>-</v>
       </c>
       <c r="L9" s="14" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!L33+'1. Inputs'!K33)/2=0),"-",(('1. Inputs'!L31+'1. Inputs'!K31)/2)/(('1. Inputs'!L33+'1. Inputs'!K33)/2))</f>
+        <f aca="false">IF(OR(('1. Inputs'!L34+'1. Inputs'!K34)/2=0),"-",(('1. Inputs'!L32+'1. Inputs'!K32)/2)/(('1. Inputs'!L34+'1. Inputs'!K34)/2))</f>
         <v>-</v>
       </c>
     </row>
@@ -9877,47 +10112,47 @@
         <v>170</v>
       </c>
       <c r="B12" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!B33+'1. Inputs'!B34)=0),"-",('1. Inputs'!B13-'1. Inputs'!B14)/('1. Inputs'!B33+'1. Inputs'!B34))</f>
+        <f aca="false">IF(OR(('1. Inputs'!B34+'1. Inputs'!B35)=0),"-",('1. Inputs'!B13-'1. Inputs'!B14)/('1. Inputs'!B34+'1. Inputs'!B35))</f>
         <v>-</v>
       </c>
       <c r="C12" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!C33+'1. Inputs'!C34)=0),"-",('1. Inputs'!C13-'1. Inputs'!C14)/('1. Inputs'!C33+'1. Inputs'!C34))</f>
+        <f aca="false">IF(OR(('1. Inputs'!C34+'1. Inputs'!C35)=0),"-",('1. Inputs'!C13-'1. Inputs'!C14)/('1. Inputs'!C34+'1. Inputs'!C35))</f>
         <v>-</v>
       </c>
       <c r="D12" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!D33+'1. Inputs'!D34)=0),"-",('1. Inputs'!D13-'1. Inputs'!D14)/('1. Inputs'!D33+'1. Inputs'!D34))</f>
+        <f aca="false">IF(OR(('1. Inputs'!D34+'1. Inputs'!D35)=0),"-",('1. Inputs'!D13-'1. Inputs'!D14)/('1. Inputs'!D34+'1. Inputs'!D35))</f>
         <v>-</v>
       </c>
       <c r="E12" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!E33+'1. Inputs'!E34)=0),"-",('1. Inputs'!E13-'1. Inputs'!E14)/('1. Inputs'!E33+'1. Inputs'!E34))</f>
+        <f aca="false">IF(OR(('1. Inputs'!E34+'1. Inputs'!E35)=0),"-",('1. Inputs'!E13-'1. Inputs'!E14)/('1. Inputs'!E34+'1. Inputs'!E35))</f>
         <v>-</v>
       </c>
       <c r="F12" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!F33+'1. Inputs'!F34)=0),"-",('1. Inputs'!F13-'1. Inputs'!F14)/('1. Inputs'!F33+'1. Inputs'!F34))</f>
+        <f aca="false">IF(OR(('1. Inputs'!F34+'1. Inputs'!F35)=0),"-",('1. Inputs'!F13-'1. Inputs'!F14)/('1. Inputs'!F34+'1. Inputs'!F35))</f>
         <v>-</v>
       </c>
       <c r="G12" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!G33+'1. Inputs'!G34)=0),"-",('1. Inputs'!G13-'1. Inputs'!G14)/('1. Inputs'!G33+'1. Inputs'!G34))</f>
+        <f aca="false">IF(OR(('1. Inputs'!G34+'1. Inputs'!G35)=0),"-",('1. Inputs'!G13-'1. Inputs'!G14)/('1. Inputs'!G34+'1. Inputs'!G35))</f>
         <v>-</v>
       </c>
       <c r="H12" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!H33+'1. Inputs'!H34)=0),"-",('1. Inputs'!H13-'1. Inputs'!H14)/('1. Inputs'!H33+'1. Inputs'!H34))</f>
+        <f aca="false">IF(OR(('1. Inputs'!H34+'1. Inputs'!H35)=0),"-",('1. Inputs'!H13-'1. Inputs'!H14)/('1. Inputs'!H34+'1. Inputs'!H35))</f>
         <v>-</v>
       </c>
       <c r="I12" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!I33+'1. Inputs'!I34)=0),"-",('1. Inputs'!I13-'1. Inputs'!I14)/('1. Inputs'!I33+'1. Inputs'!I34))</f>
+        <f aca="false">IF(OR(('1. Inputs'!I34+'1. Inputs'!I35)=0),"-",('1. Inputs'!I13-'1. Inputs'!I14)/('1. Inputs'!I34+'1. Inputs'!I35))</f>
         <v>-</v>
       </c>
       <c r="J12" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!J33+'1. Inputs'!J34)=0),"-",('1. Inputs'!J13-'1. Inputs'!J14)/('1. Inputs'!J33+'1. Inputs'!J34))</f>
+        <f aca="false">IF(OR(('1. Inputs'!J34+'1. Inputs'!J35)=0),"-",('1. Inputs'!J13-'1. Inputs'!J14)/('1. Inputs'!J34+'1. Inputs'!J35))</f>
         <v>-</v>
       </c>
       <c r="K12" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!K33+'1. Inputs'!K34)=0),"-",('1. Inputs'!K13-'1. Inputs'!K14)/('1. Inputs'!K33+'1. Inputs'!K34))</f>
+        <f aca="false">IF(OR(('1. Inputs'!K34+'1. Inputs'!K35)=0),"-",('1. Inputs'!K13-'1. Inputs'!K14)/('1. Inputs'!K34+'1. Inputs'!K35))</f>
         <v>-</v>
       </c>
       <c r="L12" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!L33+'1. Inputs'!L34)=0),"-",('1. Inputs'!L13-'1. Inputs'!L14)/('1. Inputs'!L33+'1. Inputs'!L34))</f>
+        <f aca="false">IF(OR(('1. Inputs'!L34+'1. Inputs'!L35)=0),"-",('1. Inputs'!L13-'1. Inputs'!L14)/('1. Inputs'!L34+'1. Inputs'!L35))</f>
         <v>-</v>
       </c>
     </row>
@@ -9926,47 +10161,47 @@
         <v>171</v>
       </c>
       <c r="B13" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!B33+'1. Inputs'!B34-'1. Inputs'!B35)=0),"-",('1. Inputs'!B13-'1. Inputs'!B14)*(1-IFERROR('1. Inputs'!B17/'1. Inputs'!B16,0.25))/('1. Inputs'!B33+'1. Inputs'!B34-'1. Inputs'!B35))</f>
+        <f aca="false">IF(OR(('1. Inputs'!B34+'1. Inputs'!B35-'1. Inputs'!B36)=0),"-",('1. Inputs'!B13-'1. Inputs'!B14)*(1-IFERROR('1. Inputs'!B17/'1. Inputs'!B16,0.25))/('1. Inputs'!B34+'1. Inputs'!B35-'1. Inputs'!B36))</f>
         <v>-</v>
       </c>
       <c r="C13" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!C33+'1. Inputs'!C34-'1. Inputs'!C35)=0),"-",('1. Inputs'!C13-'1. Inputs'!C14)*(1-IFERROR('1. Inputs'!C17/'1. Inputs'!C16,0.25))/('1. Inputs'!C33+'1. Inputs'!C34-'1. Inputs'!C35))</f>
+        <f aca="false">IF(OR(('1. Inputs'!C34+'1. Inputs'!C35-'1. Inputs'!C36)=0),"-",('1. Inputs'!C13-'1. Inputs'!C14)*(1-IFERROR('1. Inputs'!C17/'1. Inputs'!C16,0.25))/('1. Inputs'!C34+'1. Inputs'!C35-'1. Inputs'!C36))</f>
         <v>-</v>
       </c>
       <c r="D13" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!D33+'1. Inputs'!D34-'1. Inputs'!D35)=0),"-",('1. Inputs'!D13-'1. Inputs'!D14)*(1-IFERROR('1. Inputs'!D17/'1. Inputs'!D16,0.25))/('1. Inputs'!D33+'1. Inputs'!D34-'1. Inputs'!D35))</f>
+        <f aca="false">IF(OR(('1. Inputs'!D34+'1. Inputs'!D35-'1. Inputs'!D36)=0),"-",('1. Inputs'!D13-'1. Inputs'!D14)*(1-IFERROR('1. Inputs'!D17/'1. Inputs'!D16,0.25))/('1. Inputs'!D34+'1. Inputs'!D35-'1. Inputs'!D36))</f>
         <v>-</v>
       </c>
       <c r="E13" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!E33+'1. Inputs'!E34-'1. Inputs'!E35)=0),"-",('1. Inputs'!E13-'1. Inputs'!E14)*(1-IFERROR('1. Inputs'!E17/'1. Inputs'!E16,0.25))/('1. Inputs'!E33+'1. Inputs'!E34-'1. Inputs'!E35))</f>
+        <f aca="false">IF(OR(('1. Inputs'!E34+'1. Inputs'!E35-'1. Inputs'!E36)=0),"-",('1. Inputs'!E13-'1. Inputs'!E14)*(1-IFERROR('1. Inputs'!E17/'1. Inputs'!E16,0.25))/('1. Inputs'!E34+'1. Inputs'!E35-'1. Inputs'!E36))</f>
         <v>-</v>
       </c>
       <c r="F13" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!F33+'1. Inputs'!F34-'1. Inputs'!F35)=0),"-",('1. Inputs'!F13-'1. Inputs'!F14)*(1-IFERROR('1. Inputs'!F17/'1. Inputs'!F16,0.25))/('1. Inputs'!F33+'1. Inputs'!F34-'1. Inputs'!F35))</f>
+        <f aca="false">IF(OR(('1. Inputs'!F34+'1. Inputs'!F35-'1. Inputs'!F36)=0),"-",('1. Inputs'!F13-'1. Inputs'!F14)*(1-IFERROR('1. Inputs'!F17/'1. Inputs'!F16,0.25))/('1. Inputs'!F34+'1. Inputs'!F35-'1. Inputs'!F36))</f>
         <v>-</v>
       </c>
       <c r="G13" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!G33+'1. Inputs'!G34-'1. Inputs'!G35)=0),"-",('1. Inputs'!G13-'1. Inputs'!G14)*(1-IFERROR('1. Inputs'!G17/'1. Inputs'!G16,0.25))/('1. Inputs'!G33+'1. Inputs'!G34-'1. Inputs'!G35))</f>
+        <f aca="false">IF(OR(('1. Inputs'!G34+'1. Inputs'!G35-'1. Inputs'!G36)=0),"-",('1. Inputs'!G13-'1. Inputs'!G14)*(1-IFERROR('1. Inputs'!G17/'1. Inputs'!G16,0.25))/('1. Inputs'!G34+'1. Inputs'!G35-'1. Inputs'!G36))</f>
         <v>-</v>
       </c>
       <c r="H13" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!H33+'1. Inputs'!H34-'1. Inputs'!H35)=0),"-",('1. Inputs'!H13-'1. Inputs'!H14)*(1-IFERROR('1. Inputs'!H17/'1. Inputs'!H16,0.25))/('1. Inputs'!H33+'1. Inputs'!H34-'1. Inputs'!H35))</f>
+        <f aca="false">IF(OR(('1. Inputs'!H34+'1. Inputs'!H35-'1. Inputs'!H36)=0),"-",('1. Inputs'!H13-'1. Inputs'!H14)*(1-IFERROR('1. Inputs'!H17/'1. Inputs'!H16,0.25))/('1. Inputs'!H34+'1. Inputs'!H35-'1. Inputs'!H36))</f>
         <v>-</v>
       </c>
       <c r="I13" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!I33+'1. Inputs'!I34-'1. Inputs'!I35)=0),"-",('1. Inputs'!I13-'1. Inputs'!I14)*(1-IFERROR('1. Inputs'!I17/'1. Inputs'!I16,0.25))/('1. Inputs'!I33+'1. Inputs'!I34-'1. Inputs'!I35))</f>
+        <f aca="false">IF(OR(('1. Inputs'!I34+'1. Inputs'!I35-'1. Inputs'!I36)=0),"-",('1. Inputs'!I13-'1. Inputs'!I14)*(1-IFERROR('1. Inputs'!I17/'1. Inputs'!I16,0.25))/('1. Inputs'!I34+'1. Inputs'!I35-'1. Inputs'!I36))</f>
         <v>-</v>
       </c>
       <c r="J13" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!J33+'1. Inputs'!J34-'1. Inputs'!J35)=0),"-",('1. Inputs'!J13-'1. Inputs'!J14)*(1-IFERROR('1. Inputs'!J17/'1. Inputs'!J16,0.25))/('1. Inputs'!J33+'1. Inputs'!J34-'1. Inputs'!J35))</f>
+        <f aca="false">IF(OR(('1. Inputs'!J34+'1. Inputs'!J35-'1. Inputs'!J36)=0),"-",('1. Inputs'!J13-'1. Inputs'!J14)*(1-IFERROR('1. Inputs'!J17/'1. Inputs'!J16,0.25))/('1. Inputs'!J34+'1. Inputs'!J35-'1. Inputs'!J36))</f>
         <v>-</v>
       </c>
       <c r="K13" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!K33+'1. Inputs'!K34-'1. Inputs'!K35)=0),"-",('1. Inputs'!K13-'1. Inputs'!K14)*(1-IFERROR('1. Inputs'!K17/'1. Inputs'!K16,0.25))/('1. Inputs'!K33+'1. Inputs'!K34-'1. Inputs'!K35))</f>
+        <f aca="false">IF(OR(('1. Inputs'!K34+'1. Inputs'!K35-'1. Inputs'!K36)=0),"-",('1. Inputs'!K13-'1. Inputs'!K14)*(1-IFERROR('1. Inputs'!K17/'1. Inputs'!K16,0.25))/('1. Inputs'!K34+'1. Inputs'!K35-'1. Inputs'!K36))</f>
         <v>-</v>
       </c>
       <c r="L13" s="12" t="str">
-        <f aca="false">IF(OR(('1. Inputs'!L33+'1. Inputs'!L34-'1. Inputs'!L35)=0),"-",('1. Inputs'!L13-'1. Inputs'!L14)*(1-IFERROR('1. Inputs'!L17/'1. Inputs'!L16,0.25))/('1. Inputs'!L33+'1. Inputs'!L34-'1. Inputs'!L35))</f>
+        <f aca="false">IF(OR(('1. Inputs'!L34+'1. Inputs'!L35-'1. Inputs'!L36)=0),"-",('1. Inputs'!L13-'1. Inputs'!L14)*(1-IFERROR('1. Inputs'!L17/'1. Inputs'!L16,0.25))/('1. Inputs'!L34+'1. Inputs'!L35-'1. Inputs'!L36))</f>
         <v>-</v>
       </c>
     </row>
@@ -10405,47 +10640,47 @@
         <v>179</v>
       </c>
       <c r="B11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!B12=0,'1. Inputs'!B12=""),"-",ABS('1. Inputs'!B54)/'1. Inputs'!B12)</f>
+        <f aca="false">IF(OR('1. Inputs'!B12=0,'1. Inputs'!B12=""),"-",ABS('1. Inputs'!B55)/'1. Inputs'!B12)</f>
         <v>-</v>
       </c>
       <c r="C11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!C12=0,'1. Inputs'!C12=""),"-",ABS('1. Inputs'!C54)/'1. Inputs'!C12)</f>
+        <f aca="false">IF(OR('1. Inputs'!C12=0,'1. Inputs'!C12=""),"-",ABS('1. Inputs'!C55)/'1. Inputs'!C12)</f>
         <v>-</v>
       </c>
       <c r="D11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!D12=0,'1. Inputs'!D12=""),"-",ABS('1. Inputs'!D54)/'1. Inputs'!D12)</f>
+        <f aca="false">IF(OR('1. Inputs'!D12=0,'1. Inputs'!D12=""),"-",ABS('1. Inputs'!D55)/'1. Inputs'!D12)</f>
         <v>-</v>
       </c>
       <c r="E11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!E12=0,'1. Inputs'!E12=""),"-",ABS('1. Inputs'!E54)/'1. Inputs'!E12)</f>
+        <f aca="false">IF(OR('1. Inputs'!E12=0,'1. Inputs'!E12=""),"-",ABS('1. Inputs'!E55)/'1. Inputs'!E12)</f>
         <v>-</v>
       </c>
       <c r="F11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!F12=0,'1. Inputs'!F12=""),"-",ABS('1. Inputs'!F54)/'1. Inputs'!F12)</f>
+        <f aca="false">IF(OR('1. Inputs'!F12=0,'1. Inputs'!F12=""),"-",ABS('1. Inputs'!F55)/'1. Inputs'!F12)</f>
         <v>-</v>
       </c>
       <c r="G11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!G12=0,'1. Inputs'!G12=""),"-",ABS('1. Inputs'!G54)/'1. Inputs'!G12)</f>
+        <f aca="false">IF(OR('1. Inputs'!G12=0,'1. Inputs'!G12=""),"-",ABS('1. Inputs'!G55)/'1. Inputs'!G12)</f>
         <v>-</v>
       </c>
       <c r="H11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!H12=0,'1. Inputs'!H12=""),"-",ABS('1. Inputs'!H54)/'1. Inputs'!H12)</f>
+        <f aca="false">IF(OR('1. Inputs'!H12=0,'1. Inputs'!H12=""),"-",ABS('1. Inputs'!H55)/'1. Inputs'!H12)</f>
         <v>-</v>
       </c>
       <c r="I11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!I12=0,'1. Inputs'!I12=""),"-",ABS('1. Inputs'!I54)/'1. Inputs'!I12)</f>
+        <f aca="false">IF(OR('1. Inputs'!I12=0,'1. Inputs'!I12=""),"-",ABS('1. Inputs'!I55)/'1. Inputs'!I12)</f>
         <v>-</v>
       </c>
       <c r="J11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!J12=0,'1. Inputs'!J12=""),"-",ABS('1. Inputs'!J54)/'1. Inputs'!J12)</f>
+        <f aca="false">IF(OR('1. Inputs'!J12=0,'1. Inputs'!J12=""),"-",ABS('1. Inputs'!J55)/'1. Inputs'!J12)</f>
         <v>-</v>
       </c>
       <c r="K11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!K12=0,'1. Inputs'!K12=""),"-",ABS('1. Inputs'!K54)/'1. Inputs'!K12)</f>
+        <f aca="false">IF(OR('1. Inputs'!K12=0,'1. Inputs'!K12=""),"-",ABS('1. Inputs'!K55)/'1. Inputs'!K12)</f>
         <v>-</v>
       </c>
       <c r="L11" s="12" t="str">
-        <f aca="false">IF(OR('1. Inputs'!L12=0,'1. Inputs'!L12=""),"-",ABS('1. Inputs'!L54)/'1. Inputs'!L12)</f>
+        <f aca="false">IF(OR('1. Inputs'!L12=0,'1. Inputs'!L12=""),"-",ABS('1. Inputs'!L55)/'1. Inputs'!L12)</f>
         <v>-</v>
       </c>
     </row>
@@ -10454,47 +10689,47 @@
         <v>180</v>
       </c>
       <c r="B12" s="14" t="str">
-        <f aca="false">IF(OR('1. Inputs'!B54=0),"-",'1. Inputs'!B12/ABS('1. Inputs'!B54))</f>
+        <f aca="false">IF(OR('1. Inputs'!B55=0),"-",'1. Inputs'!B12/ABS('1. Inputs'!B55))</f>
         <v>-</v>
       </c>
       <c r="C12" s="14" t="str">
-        <f aca="false">IF(OR('1. Inputs'!C54=0),"-",'1. Inputs'!C12/ABS('1. Inputs'!C54))</f>
+        <f aca="false">IF(OR('1. Inputs'!C55=0),"-",'1. Inputs'!C12/ABS('1. Inputs'!C55))</f>
         <v>-</v>
       </c>
       <c r="D12" s="14" t="str">
-        <f aca="false">IF(OR('1. Inputs'!D54=0),"-",'1. Inputs'!D12/ABS('1. Inputs'!D54))</f>
+        <f aca="false">IF(OR('1. Inputs'!D55=0),"-",'1. Inputs'!D12/ABS('1. Inputs'!D55))</f>
         <v>-</v>
       </c>
       <c r="E12" s="14" t="str">
-        <f aca="false">IF(OR('1. Inputs'!E54=0),"-",'1. Inputs'!E12/ABS('1. Inputs'!E54))</f>
+        <f aca="false">IF(OR('1. Inputs'!E55=0),"-",'1. Inputs'!E12/ABS('1. Inputs'!E55))</f>
         <v>-</v>
       </c>
       <c r="F12" s="14" t="str">
-        <f aca="false">IF(OR('1. Inputs'!F54=0),"-",'1. Inputs'!F12/ABS('1. Inputs'!F54))</f>
+        <f aca="false">IF(OR('1. Inputs'!F55=0),"-",'1. Inputs'!F12/ABS('1. Inputs'!F55))</f>
         <v>-</v>
       </c>
       <c r="G12" s="14" t="str">
-        <f aca="false">IF(OR('1. Inputs'!G54=0),"-",'1. Inputs'!G12/ABS('1. Inputs'!G54))</f>
+        <f aca="false">IF(OR('1. Inputs'!G55=0),"-",'1. Inputs'!G12/ABS('1. Inputs'!G55))</f>
         <v>-</v>
       </c>
       <c r="H12" s="14" t="str">
-        <f aca="false">IF(OR('1. Inputs'!H54=0),"-",'1. Inputs'!H12/ABS('1. Inputs'!H54))</f>
+        <f aca="false">IF(OR('1. Inputs'!H55=0),"-",'1. Inputs'!H12/ABS('1. Inputs'!H55))</f>
         <v>-</v>
       </c>
       <c r="I12" s="14" t="str">
-        <f aca="false">IF(OR('1. Inputs'!I54=0),"-",'1. Inputs'!I12/ABS('1. Inputs'!I54))</f>
+        <f aca="false">IF(OR('1. Inputs'!I55=0),"-",'1. Inputs'!I12/ABS('1. Inputs'!I55))</f>
         <v>-</v>
       </c>
       <c r="J12" s="14" t="str">
-        <f aca="false">IF(OR('1. Inputs'!J54=0),"-",'1. Inputs'!J12/ABS('1. Inputs'!J54))</f>
+        <f aca="false">IF(OR('1. Inputs'!J55=0),"-",'1. Inputs'!J12/ABS('1. Inputs'!J55))</f>
         <v>-</v>
       </c>
       <c r="K12" s="14" t="str">
-        <f aca="false">IF(OR('1. Inputs'!K54=0),"-",'1. Inputs'!K12/ABS('1. Inputs'!K54))</f>
+        <f aca="false">IF(OR('1. Inputs'!K55=0),"-",'1. Inputs'!K12/ABS('1. Inputs'!K55))</f>
         <v>-</v>
       </c>
       <c r="L12" s="14" t="str">
-        <f aca="false">IF(OR('1. Inputs'!L54=0),"-",'1. Inputs'!L12/ABS('1. Inputs'!L54))</f>
+        <f aca="false">IF(OR('1. Inputs'!L55=0),"-",'1. Inputs'!L12/ABS('1. Inputs'!L55))</f>
         <v>-</v>
       </c>
     </row>
@@ -10502,49 +10737,49 @@
       <c r="A13" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="B13" s="14" t="e">
-        <f aca="false">IF(OR('1. Inputs'!B31=0),"-",'1. Inputs'!B12/'1. Inputs'!B31)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="C13" s="14" t="e">
-        <f aca="false">IF(OR('1. Inputs'!C31=0),"-",'1. Inputs'!C12/'1. Inputs'!C31)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="D13" s="14" t="e">
-        <f aca="false">IF(OR('1. Inputs'!D31=0),"-",'1. Inputs'!D12/'1. Inputs'!D31)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="E13" s="14" t="e">
-        <f aca="false">IF(OR('1. Inputs'!E31=0),"-",'1. Inputs'!E12/'1. Inputs'!E31)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="F13" s="14" t="e">
-        <f aca="false">IF(OR('1. Inputs'!F31=0),"-",'1. Inputs'!F12/'1. Inputs'!F31)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="G13" s="14" t="e">
-        <f aca="false">IF(OR('1. Inputs'!G31=0),"-",'1. Inputs'!G12/'1. Inputs'!G31)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="H13" s="14" t="e">
-        <f aca="false">IF(OR('1. Inputs'!H31=0),"-",'1. Inputs'!H12/'1. Inputs'!H31)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="I13" s="14" t="e">
-        <f aca="false">IF(OR('1. Inputs'!I31=0),"-",'1. Inputs'!I12/'1. Inputs'!I31)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="J13" s="14" t="e">
-        <f aca="false">IF(OR('1. Inputs'!J31=0),"-",'1. Inputs'!J12/'1. Inputs'!J31)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="K13" s="14" t="e">
-        <f aca="false">IF(OR('1. Inputs'!K31=0),"-",'1. Inputs'!K12/'1. Inputs'!K31)</f>
-        <v>#VALUE!</v>
-      </c>
-      <c r="L13" s="14" t="e">
-        <f aca="false">IF(OR('1. Inputs'!L31=0),"-",'1. Inputs'!L12/'1. Inputs'!L31)</f>
-        <v>#VALUE!</v>
+      <c r="B13" s="14" t="str">
+        <f aca="false">IF(OR('1. Inputs'!B32=0),"-",'1. Inputs'!B12/'1. Inputs'!B32)</f>
+        <v>-</v>
+      </c>
+      <c r="C13" s="14" t="str">
+        <f aca="false">IF(OR('1. Inputs'!C32=0),"-",'1. Inputs'!C12/'1. Inputs'!C32)</f>
+        <v>-</v>
+      </c>
+      <c r="D13" s="14" t="str">
+        <f aca="false">IF(OR('1. Inputs'!D32=0),"-",'1. Inputs'!D12/'1. Inputs'!D32)</f>
+        <v>-</v>
+      </c>
+      <c r="E13" s="14" t="str">
+        <f aca="false">IF(OR('1. Inputs'!E32=0),"-",'1. Inputs'!E12/'1. Inputs'!E32)</f>
+        <v>-</v>
+      </c>
+      <c r="F13" s="14" t="str">
+        <f aca="false">IF(OR('1. Inputs'!F32=0),"-",'1. Inputs'!F12/'1. Inputs'!F32)</f>
+        <v>-</v>
+      </c>
+      <c r="G13" s="14" t="str">
+        <f aca="false">IF(OR('1. Inputs'!G32=0),"-",'1. Inputs'!G12/'1. Inputs'!G32)</f>
+        <v>-</v>
+      </c>
+      <c r="H13" s="14" t="str">
+        <f aca="false">IF(OR('1. Inputs'!H32=0),"-",'1. Inputs'!H12/'1. Inputs'!H32)</f>
+        <v>-</v>
+      </c>
+      <c r="I13" s="14" t="str">
+        <f aca="false">IF(OR('1. Inputs'!I32=0),"-",'1. Inputs'!I12/'1. Inputs'!I32)</f>
+        <v>-</v>
+      </c>
+      <c r="J13" s="14" t="str">
+        <f aca="false">IF(OR('1. Inputs'!J32=0),"-",'1. Inputs'!J12/'1. Inputs'!J32)</f>
+        <v>-</v>
+      </c>
+      <c r="K13" s="14" t="str">
+        <f aca="false">IF(OR('1. Inputs'!K32=0),"-",'1. Inputs'!K12/'1. Inputs'!K32)</f>
+        <v>-</v>
+      </c>
+      <c r="L13" s="14" t="str">
+        <f aca="false">IF(OR('1. Inputs'!L32=0),"-",'1. Inputs'!L12/'1. Inputs'!L32)</f>
+        <v>-</v>
       </c>
     </row>
   </sheetData>
@@ -10766,7 +11001,7 @@
         <v>207</v>
       </c>
       <c r="B9" s="11" t="n">
-        <f aca="false">'1. Inputs'!L38</f>
+        <f aca="false">'1. Inputs'!L39</f>
         <v>0</v>
       </c>
       <c r="C9" s="18" t="s">
@@ -10777,9 +11012,9 @@
       <c r="A10" s="17" t="s">
         <v>209</v>
       </c>
-      <c r="B10" s="11" t="e">
-        <f aca="false">'1. Inputs'!L53+'1. Inputs'!L54</f>
-        <v>#VALUE!</v>
+      <c r="B10" s="11" t="n">
+        <f aca="false">'1. Inputs'!L54+'1. Inputs'!L55</f>
+        <v>0</v>
       </c>
       <c r="C10" s="18" t="s">
         <v>210</v>
@@ -10826,7 +11061,7 @@
         <v>217</v>
       </c>
       <c r="B14" s="19" t="str">
-        <f aca="false">IF(OR('1. Inputs'!L38=0,'1. Inputs'!L38=""),"-",'1. Inputs'!B4/'1. Inputs'!L38)</f>
+        <f aca="false">IF(OR('1. Inputs'!L39=0,'1. Inputs'!L39=""),"-",'1. Inputs'!B4/'1. Inputs'!L39)</f>
         <v>-</v>
       </c>
       <c r="C14" s="18" t="s">
@@ -10837,9 +11072,9 @@
       <c r="A15" s="17" t="s">
         <v>219</v>
       </c>
-      <c r="B15" s="19" t="e">
-        <f aca="false">IF(OR(('1. Inputs'!L53+'1. Inputs'!L54)=0),"-",('1. Inputs'!B4*'1. Inputs'!B5)/('1. Inputs'!L53+'1. Inputs'!L54))</f>
-        <v>#VALUE!</v>
+      <c r="B15" s="19" t="str">
+        <f aca="false">IF(OR(('1. Inputs'!L54+'1. Inputs'!L55)=0),"-",('1. Inputs'!B4*'1. Inputs'!B5)/('1. Inputs'!L54+'1. Inputs'!L55))</f>
+        <v>-</v>
       </c>
       <c r="C15" s="18" t="s">
         <v>220</v>
@@ -10850,7 +11085,7 @@
         <v>221</v>
       </c>
       <c r="B16" s="19" t="str">
-        <f aca="false">IF(OR('1. Inputs'!L13=0,'1. Inputs'!L13=""),"-",('1. Inputs'!B4*'1. Inputs'!B5+'1. Inputs'!L34-'1. Inputs'!L35)/'1. Inputs'!L13)</f>
+        <f aca="false">IF(OR('1. Inputs'!L13=0,'1. Inputs'!L13=""),"-",('1. Inputs'!B4*'1. Inputs'!B5+'1. Inputs'!L35-'1. Inputs'!L36)/'1. Inputs'!L13)</f>
         <v>-</v>
       </c>
       <c r="C16" s="18" t="s">
@@ -10874,7 +11109,7 @@
         <v>225</v>
       </c>
       <c r="B18" s="20" t="str">
-        <f aca="false">IF(OR('1. Inputs'!B4=0),"-",('1. Inputs'!L53+'1. Inputs'!L54)/('1. Inputs'!B4*'1. Inputs'!B5))</f>
+        <f aca="false">IF(OR('1. Inputs'!B4=0),"-",('1. Inputs'!L54+'1. Inputs'!L55)/('1. Inputs'!B4*'1. Inputs'!B5))</f>
         <v>-</v>
       </c>
       <c r="C18" s="18" t="s">
@@ -10910,7 +11145,7 @@
         <v>231</v>
       </c>
       <c r="B21" s="11" t="n">
-        <f aca="false">'1. Inputs'!B4*'1. Inputs'!B5+'1. Inputs'!L34-'1. Inputs'!L35</f>
+        <f aca="false">'1. Inputs'!B4*'1. Inputs'!B5+'1. Inputs'!L35-'1. Inputs'!L36</f>
         <v>0</v>
       </c>
       <c r="C21" s="18" t="s">

</xml_diff>